<commit_message>
Price 4GB laptop/desktop RAM and add DDR3-1600 group
Desktop matches laptop pricing. Adds DDR3-1600 / PC3-12800 rows
(4GB and 8GB, desktop/laptop/server).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BFknSiXKDWdHdxsn9XQpko
</commit_message>
<xml_diff>
--- a/ram_bulk_pricing.xlsx
+++ b/ram_bulk_pricing.xlsx
@@ -12,7 +12,7 @@
     <sheet name="How to use" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Bulk Pricing'!$A$4:$I$58</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Bulk Pricing'!$A$4:$I$64</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="38">
   <si>
     <t xml:space="preserve">RAM Bulk Buyer Pricing (all brands, non-gaming)</t>
   </si>
@@ -102,6 +102,9 @@
     <t xml:space="preserve">Server RDIMM (Registered ECC)</t>
   </si>
   <si>
+    <t xml:space="preserve">DDR3-1600 / PC3-12800</t>
+  </si>
+  <si>
     <t xml:space="preserve">DDR4</t>
   </si>
   <si>
@@ -129,6 +132,9 @@
     <t xml:space="preserve">Prices are per single stick, any brand, tested. Gaming RAM is NOT on this sheet; it is listed separately.</t>
   </si>
   <si>
+    <t xml:space="preserve">Desktop prices match laptop prices for the same speed and size. Server prices are set separately.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Rows are grouped by speed; the shading alternates between speed groups.</t>
   </si>
   <si>
@@ -147,7 +153,7 @@
     <t xml:space="preserve">Speed reference</t>
   </si>
   <si>
-    <t xml:space="preserve">DDR3-1333 = PC3-10600 (U = desktop, S = laptop, R = server)</t>
+    <t xml:space="preserve">DDR3-1333 = PC3-10600   DDR3-1600 = PC3-12800 (U = desktop, S = laptop, R = server)</t>
   </si>
   <si>
     <t xml:space="preserve">DDR4-2133 = PC4-17000 (2133P)   DDR4-2400 = PC4-19200 (2400T)</t>
@@ -708,7 +714,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I58"/>
+  <dimension ref="A1:I64"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
@@ -731,7 +737,9 @@
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3"/>
+      <c r="B2" s="3" t="n">
+        <v>46313</v>
+      </c>
       <c r="D2" s="4" t="s">
         <v>2</v>
       </c>
@@ -789,10 +797,12 @@
       <c r="D5" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="10"/>
-      <c r="F5" s="11" t="str">
+      <c r="E5" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="F5" s="11" t="n">
         <f aca="false">IF(E5="","",E5/C5)</f>
-        <v/>
+        <v>1.75</v>
       </c>
       <c r="G5" s="12"/>
       <c r="H5" s="11" t="str">
@@ -814,10 +824,12 @@
       <c r="D6" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="E6" s="10"/>
-      <c r="F6" s="11" t="str">
+      <c r="E6" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="F6" s="11" t="n">
         <f aca="false">IF(E6="","",E6/C6)</f>
-        <v/>
+        <v>1.75</v>
       </c>
       <c r="G6" s="12"/>
       <c r="H6" s="11" t="str">
@@ -928,10 +940,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" s="14" t="s">
         <v>18</v>
-      </c>
-      <c r="B11" s="14" t="s">
-        <v>19</v>
       </c>
       <c r="C11" s="15" t="n">
         <v>4</v>
@@ -939,10 +951,12 @@
       <c r="D11" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="E11" s="10"/>
-      <c r="F11" s="16" t="str">
+      <c r="E11" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="F11" s="16" t="n">
         <f aca="false">IF(E11="","",E11/C11)</f>
-        <v/>
+        <v>1.75</v>
       </c>
       <c r="G11" s="12"/>
       <c r="H11" s="16" t="str">
@@ -953,10 +967,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" s="14" t="s">
         <v>18</v>
-      </c>
-      <c r="B12" s="14" t="s">
-        <v>19</v>
       </c>
       <c r="C12" s="15" t="n">
         <v>4</v>
@@ -964,10 +978,12 @@
       <c r="D12" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="E12" s="10"/>
-      <c r="F12" s="16" t="str">
+      <c r="E12" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="F12" s="16" t="n">
         <f aca="false">IF(E12="","",E12/C12)</f>
-        <v/>
+        <v>1.75</v>
       </c>
       <c r="G12" s="12"/>
       <c r="H12" s="16" t="str">
@@ -978,10 +994,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" s="14" t="s">
         <v>18</v>
-      </c>
-      <c r="B13" s="14" t="s">
-        <v>19</v>
       </c>
       <c r="C13" s="15" t="n">
         <v>4</v>
@@ -1003,10 +1019,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="14" t="s">
         <v>18</v>
-      </c>
-      <c r="B14" s="14" t="s">
-        <v>19</v>
       </c>
       <c r="C14" s="15" t="n">
         <v>8</v>
@@ -1028,10 +1044,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" s="14" t="s">
         <v>18</v>
-      </c>
-      <c r="B15" s="14" t="s">
-        <v>19</v>
       </c>
       <c r="C15" s="15" t="n">
         <v>8</v>
@@ -1053,10 +1069,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B16" s="14" t="s">
         <v>18</v>
-      </c>
-      <c r="B16" s="14" t="s">
-        <v>19</v>
       </c>
       <c r="C16" s="15" t="n">
         <v>8</v>
@@ -1077,150 +1093,154 @@
       <c r="I16" s="12"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="B17" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="C17" s="15" t="n">
-        <v>16</v>
-      </c>
-      <c r="D17" s="14" t="s">
+      <c r="A17" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C17" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="D17" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E17" s="10"/>
-      <c r="F17" s="16" t="str">
+      <c r="E17" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="F17" s="11" t="n">
         <f aca="false">IF(E17="","",E17/C17)</f>
-        <v/>
+        <v>2.75</v>
       </c>
       <c r="G17" s="12"/>
-      <c r="H17" s="16" t="str">
+      <c r="H17" s="11" t="str">
         <f aca="false">IF(OR(E17="",G17=""),"",E17*G17)</f>
         <v/>
       </c>
       <c r="I17" s="12"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="B18" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="C18" s="15" t="n">
-        <v>16</v>
-      </c>
-      <c r="D18" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="E18" s="10"/>
-      <c r="F18" s="16" t="str">
+      <c r="A18" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C18" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E18" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="F18" s="11" t="n">
         <f aca="false">IF(E18="","",E18/C18)</f>
-        <v/>
+        <v>2.75</v>
       </c>
       <c r="G18" s="12"/>
-      <c r="H18" s="16" t="str">
+      <c r="H18" s="11" t="str">
         <f aca="false">IF(OR(E18="",G18=""),"",E18*G18)</f>
         <v/>
       </c>
       <c r="I18" s="12"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="B19" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="C19" s="15" t="n">
-        <v>16</v>
-      </c>
-      <c r="D19" s="14" t="s">
+      <c r="A19" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C19" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="D19" s="8" t="s">
         <v>17</v>
       </c>
       <c r="E19" s="10"/>
-      <c r="F19" s="16" t="str">
+      <c r="F19" s="11" t="str">
         <f aca="false">IF(E19="","",E19/C19)</f>
         <v/>
       </c>
       <c r="G19" s="12"/>
-      <c r="H19" s="16" t="str">
+      <c r="H19" s="11" t="str">
         <f aca="false">IF(OR(E19="",G19=""),"",E19*G19)</f>
         <v/>
       </c>
       <c r="I19" s="12"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="B20" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="C20" s="15" t="n">
-        <v>32</v>
-      </c>
-      <c r="D20" s="14" t="s">
+      <c r="A20" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C20" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="D20" s="8" t="s">
         <v>15</v>
       </c>
       <c r="E20" s="10"/>
-      <c r="F20" s="16" t="str">
+      <c r="F20" s="11" t="str">
         <f aca="false">IF(E20="","",E20/C20)</f>
         <v/>
       </c>
       <c r="G20" s="12"/>
-      <c r="H20" s="16" t="str">
+      <c r="H20" s="11" t="str">
         <f aca="false">IF(OR(E20="",G20=""),"",E20*G20)</f>
         <v/>
       </c>
       <c r="I20" s="12"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="B21" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="C21" s="15" t="n">
-        <v>32</v>
-      </c>
-      <c r="D21" s="14" t="s">
+      <c r="A21" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C21" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="D21" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E21" s="10"/>
-      <c r="F21" s="16" t="str">
+      <c r="F21" s="11" t="str">
         <f aca="false">IF(E21="","",E21/C21)</f>
         <v/>
       </c>
       <c r="G21" s="12"/>
-      <c r="H21" s="16" t="str">
+      <c r="H21" s="11" t="str">
         <f aca="false">IF(OR(E21="",G21=""),"",E21*G21)</f>
         <v/>
       </c>
       <c r="I21" s="12"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="B22" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="C22" s="15" t="n">
-        <v>32</v>
-      </c>
-      <c r="D22" s="14" t="s">
+      <c r="A22" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C22" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="D22" s="8" t="s">
         <v>17</v>
       </c>
       <c r="E22" s="10"/>
-      <c r="F22" s="16" t="str">
+      <c r="F22" s="11" t="str">
         <f aca="false">IF(E22="","",E22/C22)</f>
         <v/>
       </c>
       <c r="G22" s="12"/>
-      <c r="H22" s="16" t="str">
+      <c r="H22" s="11" t="str">
         <f aca="false">IF(OR(E22="",G22=""),"",E22*G22)</f>
         <v/>
       </c>
@@ -1228,13 +1248,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B23" s="8" t="s">
         <v>20</v>
       </c>
       <c r="C23" s="9" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="D23" s="8" t="s">
         <v>15</v>
@@ -1253,13 +1273,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B24" s="8" t="s">
         <v>20</v>
       </c>
       <c r="C24" s="9" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="D24" s="8" t="s">
         <v>16</v>
@@ -1278,13 +1298,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B25" s="8" t="s">
         <v>20</v>
       </c>
       <c r="C25" s="9" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="D25" s="8" t="s">
         <v>17</v>
@@ -1303,13 +1323,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B26" s="8" t="s">
         <v>20</v>
       </c>
       <c r="C26" s="9" t="n">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="D26" s="8" t="s">
         <v>15</v>
@@ -1328,13 +1348,13 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B27" s="8" t="s">
         <v>20</v>
       </c>
       <c r="C27" s="9" t="n">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="D27" s="8" t="s">
         <v>16</v>
@@ -1353,13 +1373,13 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B28" s="8" t="s">
         <v>20</v>
       </c>
       <c r="C28" s="9" t="n">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="D28" s="8" t="s">
         <v>17</v>
@@ -1377,150 +1397,154 @@
       <c r="I28" s="12"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B29" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="C29" s="9" t="n">
-        <v>16</v>
-      </c>
-      <c r="D29" s="8" t="s">
+      <c r="A29" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B29" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C29" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D29" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="E29" s="10"/>
-      <c r="F29" s="11" t="str">
+      <c r="E29" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="F29" s="16" t="n">
         <f aca="false">IF(E29="","",E29/C29)</f>
-        <v/>
+        <v>2.75</v>
       </c>
       <c r="G29" s="12"/>
-      <c r="H29" s="11" t="str">
+      <c r="H29" s="16" t="str">
         <f aca="false">IF(OR(E29="",G29=""),"",E29*G29)</f>
         <v/>
       </c>
       <c r="I29" s="12"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B30" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="C30" s="9" t="n">
-        <v>16</v>
-      </c>
-      <c r="D30" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="E30" s="10"/>
-      <c r="F30" s="11" t="str">
+      <c r="A30" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B30" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C30" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D30" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="E30" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="F30" s="16" t="n">
         <f aca="false">IF(E30="","",E30/C30)</f>
-        <v/>
+        <v>2.75</v>
       </c>
       <c r="G30" s="12"/>
-      <c r="H30" s="11" t="str">
+      <c r="H30" s="16" t="str">
         <f aca="false">IF(OR(E30="",G30=""),"",E30*G30)</f>
         <v/>
       </c>
       <c r="I30" s="12"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B31" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="C31" s="9" t="n">
-        <v>16</v>
-      </c>
-      <c r="D31" s="8" t="s">
+      <c r="A31" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B31" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C31" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D31" s="14" t="s">
         <v>17</v>
       </c>
       <c r="E31" s="10"/>
-      <c r="F31" s="11" t="str">
+      <c r="F31" s="16" t="str">
         <f aca="false">IF(E31="","",E31/C31)</f>
         <v/>
       </c>
       <c r="G31" s="12"/>
-      <c r="H31" s="11" t="str">
+      <c r="H31" s="16" t="str">
         <f aca="false">IF(OR(E31="",G31=""),"",E31*G31)</f>
         <v/>
       </c>
       <c r="I31" s="12"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B32" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="C32" s="9" t="n">
-        <v>32</v>
-      </c>
-      <c r="D32" s="8" t="s">
+      <c r="A32" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B32" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C32" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="D32" s="14" t="s">
         <v>15</v>
       </c>
       <c r="E32" s="10"/>
-      <c r="F32" s="11" t="str">
+      <c r="F32" s="16" t="str">
         <f aca="false">IF(E32="","",E32/C32)</f>
         <v/>
       </c>
       <c r="G32" s="12"/>
-      <c r="H32" s="11" t="str">
+      <c r="H32" s="16" t="str">
         <f aca="false">IF(OR(E32="",G32=""),"",E32*G32)</f>
         <v/>
       </c>
       <c r="I32" s="12"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B33" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="C33" s="9" t="n">
-        <v>32</v>
-      </c>
-      <c r="D33" s="8" t="s">
+      <c r="A33" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B33" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C33" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="D33" s="14" t="s">
         <v>16</v>
       </c>
       <c r="E33" s="10"/>
-      <c r="F33" s="11" t="str">
+      <c r="F33" s="16" t="str">
         <f aca="false">IF(E33="","",E33/C33)</f>
         <v/>
       </c>
       <c r="G33" s="12"/>
-      <c r="H33" s="11" t="str">
+      <c r="H33" s="16" t="str">
         <f aca="false">IF(OR(E33="",G33=""),"",E33*G33)</f>
         <v/>
       </c>
       <c r="I33" s="12"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B34" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="C34" s="9" t="n">
-        <v>32</v>
-      </c>
-      <c r="D34" s="8" t="s">
+      <c r="A34" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B34" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C34" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="D34" s="14" t="s">
         <v>17</v>
       </c>
       <c r="E34" s="10"/>
-      <c r="F34" s="11" t="str">
+      <c r="F34" s="16" t="str">
         <f aca="false">IF(E34="","",E34/C34)</f>
         <v/>
       </c>
       <c r="G34" s="12"/>
-      <c r="H34" s="11" t="str">
+      <c r="H34" s="16" t="str">
         <f aca="false">IF(OR(E34="",G34=""),"",E34*G34)</f>
         <v/>
       </c>
@@ -1528,13 +1552,13 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B35" s="14" t="s">
         <v>21</v>
       </c>
       <c r="C35" s="15" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="D35" s="14" t="s">
         <v>15</v>
@@ -1553,13 +1577,13 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B36" s="14" t="s">
         <v>21</v>
       </c>
       <c r="C36" s="15" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="D36" s="14" t="s">
         <v>16</v>
@@ -1578,13 +1602,13 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B37" s="14" t="s">
         <v>21</v>
       </c>
       <c r="C37" s="15" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="D37" s="14" t="s">
         <v>17</v>
@@ -1603,13 +1627,13 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B38" s="14" t="s">
         <v>21</v>
       </c>
       <c r="C38" s="15" t="n">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="D38" s="14" t="s">
         <v>15</v>
@@ -1628,13 +1652,13 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B39" s="14" t="s">
         <v>21</v>
       </c>
       <c r="C39" s="15" t="n">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="D39" s="14" t="s">
         <v>16</v>
@@ -1653,13 +1677,13 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B40" s="14" t="s">
         <v>21</v>
       </c>
       <c r="C40" s="15" t="n">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="D40" s="14" t="s">
         <v>17</v>
@@ -1677,150 +1701,154 @@
       <c r="I40" s="12"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="B41" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="C41" s="15" t="n">
-        <v>16</v>
-      </c>
-      <c r="D41" s="14" t="s">
+      <c r="A41" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B41" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C41" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="D41" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E41" s="10"/>
-      <c r="F41" s="16" t="str">
+      <c r="E41" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="F41" s="11" t="n">
         <f aca="false">IF(E41="","",E41/C41)</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="G41" s="12"/>
-      <c r="H41" s="16" t="str">
+      <c r="H41" s="11" t="str">
         <f aca="false">IF(OR(E41="",G41=""),"",E41*G41)</f>
         <v/>
       </c>
       <c r="I41" s="12"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="B42" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="C42" s="15" t="n">
-        <v>16</v>
-      </c>
-      <c r="D42" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="E42" s="10"/>
-      <c r="F42" s="16" t="str">
+      <c r="A42" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B42" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C42" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="D42" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E42" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="F42" s="11" t="n">
         <f aca="false">IF(E42="","",E42/C42)</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="G42" s="12"/>
-      <c r="H42" s="16" t="str">
+      <c r="H42" s="11" t="str">
         <f aca="false">IF(OR(E42="",G42=""),"",E42*G42)</f>
         <v/>
       </c>
       <c r="I42" s="12"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="B43" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="C43" s="15" t="n">
-        <v>16</v>
-      </c>
-      <c r="D43" s="14" t="s">
+      <c r="A43" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B43" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C43" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="D43" s="8" t="s">
         <v>17</v>
       </c>
       <c r="E43" s="10"/>
-      <c r="F43" s="16" t="str">
+      <c r="F43" s="11" t="str">
         <f aca="false">IF(E43="","",E43/C43)</f>
         <v/>
       </c>
       <c r="G43" s="12"/>
-      <c r="H43" s="16" t="str">
+      <c r="H43" s="11" t="str">
         <f aca="false">IF(OR(E43="",G43=""),"",E43*G43)</f>
         <v/>
       </c>
       <c r="I43" s="12"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="B44" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="C44" s="15" t="n">
-        <v>32</v>
-      </c>
-      <c r="D44" s="14" t="s">
+      <c r="A44" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B44" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C44" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="D44" s="8" t="s">
         <v>15</v>
       </c>
       <c r="E44" s="10"/>
-      <c r="F44" s="16" t="str">
+      <c r="F44" s="11" t="str">
         <f aca="false">IF(E44="","",E44/C44)</f>
         <v/>
       </c>
       <c r="G44" s="12"/>
-      <c r="H44" s="16" t="str">
+      <c r="H44" s="11" t="str">
         <f aca="false">IF(OR(E44="",G44=""),"",E44*G44)</f>
         <v/>
       </c>
       <c r="I44" s="12"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="B45" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="C45" s="15" t="n">
-        <v>32</v>
-      </c>
-      <c r="D45" s="14" t="s">
+      <c r="A45" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B45" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C45" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="D45" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E45" s="10"/>
-      <c r="F45" s="16" t="str">
+      <c r="F45" s="11" t="str">
         <f aca="false">IF(E45="","",E45/C45)</f>
         <v/>
       </c>
       <c r="G45" s="12"/>
-      <c r="H45" s="16" t="str">
+      <c r="H45" s="11" t="str">
         <f aca="false">IF(OR(E45="",G45=""),"",E45*G45)</f>
         <v/>
       </c>
       <c r="I45" s="12"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="B46" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="C46" s="15" t="n">
-        <v>32</v>
-      </c>
-      <c r="D46" s="14" t="s">
+      <c r="A46" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B46" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C46" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="D46" s="8" t="s">
         <v>17</v>
       </c>
       <c r="E46" s="10"/>
-      <c r="F46" s="16" t="str">
+      <c r="F46" s="11" t="str">
         <f aca="false">IF(E46="","",E46/C46)</f>
         <v/>
       </c>
       <c r="G46" s="12"/>
-      <c r="H46" s="16" t="str">
+      <c r="H46" s="11" t="str">
         <f aca="false">IF(OR(E46="",G46=""),"",E46*G46)</f>
         <v/>
       </c>
@@ -1828,13 +1856,13 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B47" s="8" t="s">
         <v>22</v>
       </c>
       <c r="C47" s="9" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="D47" s="8" t="s">
         <v>15</v>
@@ -1853,13 +1881,13 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B48" s="8" t="s">
         <v>22</v>
       </c>
       <c r="C48" s="9" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="D48" s="8" t="s">
         <v>16</v>
@@ -1878,13 +1906,13 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B49" s="8" t="s">
         <v>22</v>
       </c>
       <c r="C49" s="9" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="D49" s="8" t="s">
         <v>17</v>
@@ -1903,13 +1931,13 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B50" s="8" t="s">
         <v>22</v>
       </c>
       <c r="C50" s="9" t="n">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="D50" s="8" t="s">
         <v>15</v>
@@ -1928,13 +1956,13 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B51" s="8" t="s">
         <v>22</v>
       </c>
       <c r="C51" s="9" t="n">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="D51" s="8" t="s">
         <v>16</v>
@@ -1953,13 +1981,13 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B52" s="8" t="s">
         <v>22</v>
       </c>
       <c r="C52" s="9" t="n">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="D52" s="8" t="s">
         <v>17</v>
@@ -1977,157 +2005,311 @@
       <c r="I52" s="12"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B53" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C53" s="9" t="n">
-        <v>16</v>
-      </c>
-      <c r="D53" s="8" t="s">
+      <c r="A53" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B53" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C53" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D53" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="E53" s="10"/>
-      <c r="F53" s="11" t="str">
+      <c r="E53" s="10" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="F53" s="16" t="n">
         <f aca="false">IF(E53="","",E53/C53)</f>
-        <v/>
+        <v>3.375</v>
       </c>
       <c r="G53" s="12"/>
-      <c r="H53" s="11" t="str">
+      <c r="H53" s="16" t="str">
         <f aca="false">IF(OR(E53="",G53=""),"",E53*G53)</f>
         <v/>
       </c>
       <c r="I53" s="12"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B54" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C54" s="9" t="n">
-        <v>16</v>
-      </c>
-      <c r="D54" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="E54" s="10"/>
-      <c r="F54" s="11" t="str">
+      <c r="A54" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B54" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C54" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D54" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="E54" s="10" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="F54" s="16" t="n">
         <f aca="false">IF(E54="","",E54/C54)</f>
-        <v/>
+        <v>3.375</v>
       </c>
       <c r="G54" s="12"/>
-      <c r="H54" s="11" t="str">
+      <c r="H54" s="16" t="str">
         <f aca="false">IF(OR(E54="",G54=""),"",E54*G54)</f>
         <v/>
       </c>
       <c r="I54" s="12"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B55" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C55" s="9" t="n">
-        <v>16</v>
-      </c>
-      <c r="D55" s="8" t="s">
+      <c r="A55" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B55" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C55" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D55" s="14" t="s">
         <v>17</v>
       </c>
       <c r="E55" s="10"/>
-      <c r="F55" s="11" t="str">
+      <c r="F55" s="16" t="str">
         <f aca="false">IF(E55="","",E55/C55)</f>
         <v/>
       </c>
       <c r="G55" s="12"/>
-      <c r="H55" s="11" t="str">
+      <c r="H55" s="16" t="str">
         <f aca="false">IF(OR(E55="",G55=""),"",E55*G55)</f>
         <v/>
       </c>
       <c r="I55" s="12"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B56" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C56" s="9" t="n">
+      <c r="A56" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B56" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C56" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="D56" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="E56" s="10"/>
+      <c r="F56" s="16" t="str">
+        <f aca="false">IF(E56="","",E56/C56)</f>
+        <v/>
+      </c>
+      <c r="G56" s="12"/>
+      <c r="H56" s="16" t="str">
+        <f aca="false">IF(OR(E56="",G56=""),"",E56*G56)</f>
+        <v/>
+      </c>
+      <c r="I56" s="12"/>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B57" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C57" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="D57" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="E57" s="10"/>
+      <c r="F57" s="16" t="str">
+        <f aca="false">IF(E57="","",E57/C57)</f>
+        <v/>
+      </c>
+      <c r="G57" s="12"/>
+      <c r="H57" s="16" t="str">
+        <f aca="false">IF(OR(E57="",G57=""),"",E57*G57)</f>
+        <v/>
+      </c>
+      <c r="I57" s="12"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B58" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C58" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="D58" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="E58" s="10"/>
+      <c r="F58" s="16" t="str">
+        <f aca="false">IF(E58="","",E58/C58)</f>
+        <v/>
+      </c>
+      <c r="G58" s="12"/>
+      <c r="H58" s="16" t="str">
+        <f aca="false">IF(OR(E58="",G58=""),"",E58*G58)</f>
+        <v/>
+      </c>
+      <c r="I58" s="12"/>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B59" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C59" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="D59" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="E59" s="10"/>
+      <c r="F59" s="16" t="str">
+        <f aca="false">IF(E59="","",E59/C59)</f>
+        <v/>
+      </c>
+      <c r="G59" s="12"/>
+      <c r="H59" s="16" t="str">
+        <f aca="false">IF(OR(E59="",G59=""),"",E59*G59)</f>
+        <v/>
+      </c>
+      <c r="I59" s="12"/>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B60" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C60" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="D60" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="E60" s="10"/>
+      <c r="F60" s="16" t="str">
+        <f aca="false">IF(E60="","",E60/C60)</f>
+        <v/>
+      </c>
+      <c r="G60" s="12"/>
+      <c r="H60" s="16" t="str">
+        <f aca="false">IF(OR(E60="",G60=""),"",E60*G60)</f>
+        <v/>
+      </c>
+      <c r="I60" s="12"/>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B61" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C61" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="D61" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="E61" s="10"/>
+      <c r="F61" s="16" t="str">
+        <f aca="false">IF(E61="","",E61/C61)</f>
+        <v/>
+      </c>
+      <c r="G61" s="12"/>
+      <c r="H61" s="16" t="str">
+        <f aca="false">IF(OR(E61="",G61=""),"",E61*G61)</f>
+        <v/>
+      </c>
+      <c r="I61" s="12"/>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B62" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C62" s="15" t="n">
         <v>32</v>
       </c>
-      <c r="D56" s="8" t="s">
+      <c r="D62" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="E56" s="10"/>
-      <c r="F56" s="11" t="str">
-        <f aca="false">IF(E56="","",E56/C56)</f>
-        <v/>
-      </c>
-      <c r="G56" s="12"/>
-      <c r="H56" s="11" t="str">
-        <f aca="false">IF(OR(E56="",G56=""),"",E56*G56)</f>
-        <v/>
-      </c>
-      <c r="I56" s="12"/>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B57" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C57" s="9" t="n">
+      <c r="E62" s="10"/>
+      <c r="F62" s="16" t="str">
+        <f aca="false">IF(E62="","",E62/C62)</f>
+        <v/>
+      </c>
+      <c r="G62" s="12"/>
+      <c r="H62" s="16" t="str">
+        <f aca="false">IF(OR(E62="",G62=""),"",E62*G62)</f>
+        <v/>
+      </c>
+      <c r="I62" s="12"/>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B63" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C63" s="15" t="n">
         <v>32</v>
       </c>
-      <c r="D57" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="E57" s="10"/>
-      <c r="F57" s="11" t="str">
-        <f aca="false">IF(E57="","",E57/C57)</f>
-        <v/>
-      </c>
-      <c r="G57" s="12"/>
-      <c r="H57" s="11" t="str">
-        <f aca="false">IF(OR(E57="",G57=""),"",E57*G57)</f>
-        <v/>
-      </c>
-      <c r="I57" s="12"/>
-    </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B58" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C58" s="9" t="n">
+      <c r="D63" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="E63" s="10"/>
+      <c r="F63" s="16" t="str">
+        <f aca="false">IF(E63="","",E63/C63)</f>
+        <v/>
+      </c>
+      <c r="G63" s="12"/>
+      <c r="H63" s="16" t="str">
+        <f aca="false">IF(OR(E63="",G63=""),"",E63*G63)</f>
+        <v/>
+      </c>
+      <c r="I63" s="12"/>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B64" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C64" s="15" t="n">
         <v>32</v>
       </c>
-      <c r="D58" s="8" t="s">
+      <c r="D64" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="E58" s="10"/>
-      <c r="F58" s="11" t="str">
-        <f aca="false">IF(E58="","",E58/C58)</f>
-        <v/>
-      </c>
-      <c r="G58" s="12"/>
-      <c r="H58" s="11" t="str">
-        <f aca="false">IF(OR(E58="",G58=""),"",E58*G58)</f>
-        <v/>
-      </c>
-      <c r="I58" s="12"/>
+      <c r="E64" s="10"/>
+      <c r="F64" s="16" t="str">
+        <f aca="false">IF(E64="","",E64/C64)</f>
+        <v/>
+      </c>
+      <c r="G64" s="12"/>
+      <c r="H64" s="16" t="str">
+        <f aca="false">IF(OR(E64="",G64=""),"",E64*G64)</f>
+        <v/>
+      </c>
+      <c r="I64" s="12"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I58"/>
+  <autoFilter ref="A4:I64"/>
   <dataValidations count="1">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:D1000" type="list">
       <formula1>"Desktop UDIMM (Non-ECC),Laptop SODIMM (Non-ECC),Server RDIMM (Registered ECC)"</formula1>
@@ -2151,7 +2333,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="110"/>
@@ -2159,7 +2341,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="17" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2167,68 +2349,73 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="18" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18"/>
+      <c r="A7" s="18" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
-        <v>28</v>
-      </c>
+      <c r="A8" s="18"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="18" t="s">
-        <v>29</v>
+      <c r="A9" s="19" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="18"/>
+      <c r="A12" s="18" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="19" t="s">
-        <v>32</v>
-      </c>
+      <c r="A13" s="18"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="18" t="s">
-        <v>33</v>
+      <c r="A14" s="19" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="s">
-        <v>35</v>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="18" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Price 4GB server RDIMMs to match desktop/laptop
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BFknSiXKDWdHdxsn9XQpko
</commit_message>
<xml_diff>
--- a/ram_bulk_pricing.xlsx
+++ b/ram_bulk_pricing.xlsx
@@ -132,7 +132,7 @@
     <t xml:space="preserve">Prices are per single stick, any brand, tested. Gaming RAM is NOT on this sheet; it is listed separately.</t>
   </si>
   <si>
-    <t xml:space="preserve">Desktop prices match laptop prices for the same speed and size. Server prices are set separately.</t>
+    <t xml:space="preserve">4GB: desktop, laptop and server are all the same price for a given speed.</t>
   </si>
   <si>
     <t xml:space="preserve">Rows are grouped by speed; the shading alternates between speed groups.</t>
@@ -851,10 +851,12 @@
       <c r="D7" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="E7" s="10"/>
-      <c r="F7" s="11" t="str">
+      <c r="E7" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="F7" s="11" t="n">
         <f aca="false">IF(E7="","",E7/C7)</f>
-        <v/>
+        <v>1.75</v>
       </c>
       <c r="G7" s="12"/>
       <c r="H7" s="11" t="str">
@@ -1005,10 +1007,12 @@
       <c r="D13" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="E13" s="10"/>
-      <c r="F13" s="16" t="str">
+      <c r="E13" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="F13" s="16" t="n">
         <f aca="false">IF(E13="","",E13/C13)</f>
-        <v/>
+        <v>1.75</v>
       </c>
       <c r="G13" s="12"/>
       <c r="H13" s="16" t="str">
@@ -1159,10 +1163,12 @@
       <c r="D19" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="E19" s="10"/>
-      <c r="F19" s="11" t="str">
+      <c r="E19" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="F19" s="11" t="n">
         <f aca="false">IF(E19="","",E19/C19)</f>
-        <v/>
+        <v>2.75</v>
       </c>
       <c r="G19" s="12"/>
       <c r="H19" s="11" t="str">
@@ -1463,10 +1469,12 @@
       <c r="D31" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="E31" s="10"/>
-      <c r="F31" s="16" t="str">
+      <c r="E31" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="F31" s="16" t="n">
         <f aca="false">IF(E31="","",E31/C31)</f>
-        <v/>
+        <v>2.75</v>
       </c>
       <c r="G31" s="12"/>
       <c r="H31" s="16" t="str">
@@ -1767,10 +1775,12 @@
       <c r="D43" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="E43" s="10"/>
-      <c r="F43" s="11" t="str">
+      <c r="E43" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="F43" s="11" t="n">
         <f aca="false">IF(E43="","",E43/C43)</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="G43" s="12"/>
       <c r="H43" s="11" t="str">
@@ -2071,10 +2081,12 @@
       <c r="D55" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="E55" s="10"/>
-      <c r="F55" s="16" t="str">
+      <c r="E55" s="10" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="F55" s="16" t="n">
         <f aca="false">IF(E55="","",E55/C55)</f>
-        <v/>
+        <v>3.375</v>
       </c>
       <c r="G55" s="12"/>
       <c r="H55" s="16" t="str">

</xml_diff>

<commit_message>
Price 8GB, 16GB and 32GB desktop/laptop RAM
8GB per owner list; DDR4 16GB = 2x8GB + $2.50, 32GB = 2x16GB + $2.50.
Server 8GB+ left blank.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BFknSiXKDWdHdxsn9XQpko
</commit_message>
<xml_diff>
--- a/ram_bulk_pricing.xlsx
+++ b/ram_bulk_pricing.xlsx
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="40">
   <si>
     <t xml:space="preserve">RAM Bulk Buyer Pricing (all brands, non-gaming)</t>
   </si>
@@ -133,6 +133,12 @@
   </si>
   <si>
     <t xml:space="preserve">4GB: desktop, laptop and server are all the same price for a given speed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8GB and up: desktop and laptop are the same price; server is priced separately.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DDR4 16GB = 2 x the 8GB price + $2.50.  DDR4 32GB = 2 x the 16GB price + $2.50.  DDR3 16/32GB not priced.</t>
   </si>
   <si>
     <t xml:space="preserve">Rows are grouped by speed; the shading alternates between speed groups.</t>
@@ -878,10 +884,12 @@
       <c r="D8" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="10"/>
-      <c r="F8" s="11" t="str">
+      <c r="E8" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="F8" s="11" t="n">
         <f aca="false">IF(E8="","",E8/C8)</f>
-        <v/>
+        <v>1.375</v>
       </c>
       <c r="G8" s="12"/>
       <c r="H8" s="11" t="str">
@@ -903,10 +911,12 @@
       <c r="D9" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="E9" s="10"/>
-      <c r="F9" s="11" t="str">
+      <c r="E9" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="F9" s="11" t="n">
         <f aca="false">IF(E9="","",E9/C9)</f>
-        <v/>
+        <v>1.375</v>
       </c>
       <c r="G9" s="12"/>
       <c r="H9" s="11" t="str">
@@ -1034,10 +1044,12 @@
       <c r="D14" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="E14" s="10"/>
-      <c r="F14" s="16" t="str">
+      <c r="E14" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="F14" s="16" t="n">
         <f aca="false">IF(E14="","",E14/C14)</f>
-        <v/>
+        <v>1.375</v>
       </c>
       <c r="G14" s="12"/>
       <c r="H14" s="16" t="str">
@@ -1059,10 +1071,12 @@
       <c r="D15" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="E15" s="10"/>
-      <c r="F15" s="16" t="str">
+      <c r="E15" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="F15" s="16" t="n">
         <f aca="false">IF(E15="","",E15/C15)</f>
-        <v/>
+        <v>1.375</v>
       </c>
       <c r="G15" s="12"/>
       <c r="H15" s="16" t="str">
@@ -1190,10 +1204,12 @@
       <c r="D20" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E20" s="10"/>
-      <c r="F20" s="11" t="str">
+      <c r="E20" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="F20" s="11" t="n">
         <f aca="false">IF(E20="","",E20/C20)</f>
-        <v/>
+        <v>2.75</v>
       </c>
       <c r="G20" s="12"/>
       <c r="H20" s="11" t="str">
@@ -1215,10 +1231,12 @@
       <c r="D21" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="E21" s="10"/>
-      <c r="F21" s="11" t="str">
+      <c r="E21" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="F21" s="11" t="n">
         <f aca="false">IF(E21="","",E21/C21)</f>
-        <v/>
+        <v>2.75</v>
       </c>
       <c r="G21" s="12"/>
       <c r="H21" s="11" t="str">
@@ -1265,10 +1283,12 @@
       <c r="D23" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E23" s="10"/>
-      <c r="F23" s="11" t="str">
+      <c r="E23" s="10" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="F23" s="11" t="n">
         <f aca="false">IF(E23="","",E23/C23)</f>
-        <v/>
+        <v>2.90625</v>
       </c>
       <c r="G23" s="12"/>
       <c r="H23" s="11" t="str">
@@ -1290,10 +1310,12 @@
       <c r="D24" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="E24" s="10"/>
-      <c r="F24" s="11" t="str">
+      <c r="E24" s="10" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="F24" s="11" t="n">
         <f aca="false">IF(E24="","",E24/C24)</f>
-        <v/>
+        <v>2.90625</v>
       </c>
       <c r="G24" s="12"/>
       <c r="H24" s="11" t="str">
@@ -1340,10 +1362,12 @@
       <c r="D26" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E26" s="10"/>
-      <c r="F26" s="11" t="str">
+      <c r="E26" s="10" t="n">
+        <v>95.5</v>
+      </c>
+      <c r="F26" s="11" t="n">
         <f aca="false">IF(E26="","",E26/C26)</f>
-        <v/>
+        <v>2.984375</v>
       </c>
       <c r="G26" s="12"/>
       <c r="H26" s="11" t="str">
@@ -1365,10 +1389,12 @@
       <c r="D27" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="E27" s="10"/>
-      <c r="F27" s="11" t="str">
+      <c r="E27" s="10" t="n">
+        <v>95.5</v>
+      </c>
+      <c r="F27" s="11" t="n">
         <f aca="false">IF(E27="","",E27/C27)</f>
-        <v/>
+        <v>2.984375</v>
       </c>
       <c r="G27" s="12"/>
       <c r="H27" s="11" t="str">
@@ -1496,10 +1522,12 @@
       <c r="D32" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="E32" s="10"/>
-      <c r="F32" s="16" t="str">
+      <c r="E32" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="F32" s="16" t="n">
         <f aca="false">IF(E32="","",E32/C32)</f>
-        <v/>
+        <v>2.75</v>
       </c>
       <c r="G32" s="12"/>
       <c r="H32" s="16" t="str">
@@ -1521,10 +1549,12 @@
       <c r="D33" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="E33" s="10"/>
-      <c r="F33" s="16" t="str">
+      <c r="E33" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="F33" s="16" t="n">
         <f aca="false">IF(E33="","",E33/C33)</f>
-        <v/>
+        <v>2.75</v>
       </c>
       <c r="G33" s="12"/>
       <c r="H33" s="16" t="str">
@@ -1571,10 +1601,12 @@
       <c r="D35" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="E35" s="10"/>
-      <c r="F35" s="16" t="str">
+      <c r="E35" s="10" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="F35" s="16" t="n">
         <f aca="false">IF(E35="","",E35/C35)</f>
-        <v/>
+        <v>2.90625</v>
       </c>
       <c r="G35" s="12"/>
       <c r="H35" s="16" t="str">
@@ -1596,10 +1628,12 @@
       <c r="D36" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="E36" s="10"/>
-      <c r="F36" s="16" t="str">
+      <c r="E36" s="10" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="F36" s="16" t="n">
         <f aca="false">IF(E36="","",E36/C36)</f>
-        <v/>
+        <v>2.90625</v>
       </c>
       <c r="G36" s="12"/>
       <c r="H36" s="16" t="str">
@@ -1646,10 +1680,12 @@
       <c r="D38" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="E38" s="10"/>
-      <c r="F38" s="16" t="str">
+      <c r="E38" s="10" t="n">
+        <v>95.5</v>
+      </c>
+      <c r="F38" s="16" t="n">
         <f aca="false">IF(E38="","",E38/C38)</f>
-        <v/>
+        <v>2.984375</v>
       </c>
       <c r="G38" s="12"/>
       <c r="H38" s="16" t="str">
@@ -1671,10 +1707,12 @@
       <c r="D39" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="E39" s="10"/>
-      <c r="F39" s="16" t="str">
+      <c r="E39" s="10" t="n">
+        <v>95.5</v>
+      </c>
+      <c r="F39" s="16" t="n">
         <f aca="false">IF(E39="","",E39/C39)</f>
-        <v/>
+        <v>2.984375</v>
       </c>
       <c r="G39" s="12"/>
       <c r="H39" s="16" t="str">
@@ -1802,10 +1840,12 @@
       <c r="D44" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E44" s="10"/>
-      <c r="F44" s="11" t="str">
+      <c r="E44" s="10" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="F44" s="11" t="n">
         <f aca="false">IF(E44="","",E44/C44)</f>
-        <v/>
+        <v>2.9375</v>
       </c>
       <c r="G44" s="12"/>
       <c r="H44" s="11" t="str">
@@ -1827,10 +1867,12 @@
       <c r="D45" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="E45" s="10"/>
-      <c r="F45" s="11" t="str">
+      <c r="E45" s="10" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="F45" s="11" t="n">
         <f aca="false">IF(E45="","",E45/C45)</f>
-        <v/>
+        <v>2.9375</v>
       </c>
       <c r="G45" s="12"/>
       <c r="H45" s="11" t="str">
@@ -1877,10 +1919,12 @@
       <c r="D47" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E47" s="10"/>
-      <c r="F47" s="11" t="str">
+      <c r="E47" s="10" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="F47" s="11" t="n">
         <f aca="false">IF(E47="","",E47/C47)</f>
-        <v/>
+        <v>3.09375</v>
       </c>
       <c r="G47" s="12"/>
       <c r="H47" s="11" t="str">
@@ -1902,10 +1946,12 @@
       <c r="D48" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="E48" s="10"/>
-      <c r="F48" s="11" t="str">
+      <c r="E48" s="10" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="F48" s="11" t="n">
         <f aca="false">IF(E48="","",E48/C48)</f>
-        <v/>
+        <v>3.09375</v>
       </c>
       <c r="G48" s="12"/>
       <c r="H48" s="11" t="str">
@@ -1952,10 +1998,12 @@
       <c r="D50" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E50" s="10"/>
-      <c r="F50" s="11" t="str">
+      <c r="E50" s="10" t="n">
+        <v>101.5</v>
+      </c>
+      <c r="F50" s="11" t="n">
         <f aca="false">IF(E50="","",E50/C50)</f>
-        <v/>
+        <v>3.171875</v>
       </c>
       <c r="G50" s="12"/>
       <c r="H50" s="11" t="str">
@@ -1977,10 +2025,12 @@
       <c r="D51" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="E51" s="10"/>
-      <c r="F51" s="11" t="str">
+      <c r="E51" s="10" t="n">
+        <v>101.5</v>
+      </c>
+      <c r="F51" s="11" t="n">
         <f aca="false">IF(E51="","",E51/C51)</f>
-        <v/>
+        <v>3.171875</v>
       </c>
       <c r="G51" s="12"/>
       <c r="H51" s="11" t="str">
@@ -2108,10 +2158,12 @@
       <c r="D56" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="E56" s="10"/>
-      <c r="F56" s="16" t="str">
+      <c r="E56" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="F56" s="16" t="n">
         <f aca="false">IF(E56="","",E56/C56)</f>
-        <v/>
+        <v>3.125</v>
       </c>
       <c r="G56" s="12"/>
       <c r="H56" s="16" t="str">
@@ -2133,10 +2185,12 @@
       <c r="D57" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="E57" s="10"/>
-      <c r="F57" s="16" t="str">
+      <c r="E57" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="F57" s="16" t="n">
         <f aca="false">IF(E57="","",E57/C57)</f>
-        <v/>
+        <v>3.125</v>
       </c>
       <c r="G57" s="12"/>
       <c r="H57" s="16" t="str">
@@ -2183,10 +2237,12 @@
       <c r="D59" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="E59" s="10"/>
-      <c r="F59" s="16" t="str">
+      <c r="E59" s="10" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="F59" s="16" t="n">
         <f aca="false">IF(E59="","",E59/C59)</f>
-        <v/>
+        <v>3.28125</v>
       </c>
       <c r="G59" s="12"/>
       <c r="H59" s="16" t="str">
@@ -2208,10 +2264,12 @@
       <c r="D60" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="E60" s="10"/>
-      <c r="F60" s="16" t="str">
+      <c r="E60" s="10" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="F60" s="16" t="n">
         <f aca="false">IF(E60="","",E60/C60)</f>
-        <v/>
+        <v>3.28125</v>
       </c>
       <c r="G60" s="12"/>
       <c r="H60" s="16" t="str">
@@ -2258,10 +2316,12 @@
       <c r="D62" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="E62" s="10"/>
-      <c r="F62" s="16" t="str">
+      <c r="E62" s="10" t="n">
+        <v>107.5</v>
+      </c>
+      <c r="F62" s="16" t="n">
         <f aca="false">IF(E62="","",E62/C62)</f>
-        <v/>
+        <v>3.359375</v>
       </c>
       <c r="G62" s="12"/>
       <c r="H62" s="16" t="str">
@@ -2283,10 +2343,12 @@
       <c r="D63" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="E63" s="10"/>
-      <c r="F63" s="16" t="str">
+      <c r="E63" s="10" t="n">
+        <v>107.5</v>
+      </c>
+      <c r="F63" s="16" t="n">
         <f aca="false">IF(E63="","",E63/C63)</f>
-        <v/>
+        <v>3.359375</v>
       </c>
       <c r="G63" s="12"/>
       <c r="H63" s="16" t="str">
@@ -2345,7 +2407,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="110"/>
@@ -2385,20 +2447,20 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="18"/>
+      <c r="A8" s="18" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="s">
-        <v>30</v>
+      <c r="A9" s="18" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="18" t="s">
-        <v>31</v>
-      </c>
+      <c r="A10" s="18"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="18" t="s">
+      <c r="A11" s="19" t="s">
         <v>32</v>
       </c>
     </row>
@@ -2408,26 +2470,36 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="18"/>
+      <c r="A13" s="18" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="19" t="s">
-        <v>34</v>
+      <c r="A14" s="18" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="18" t="s">
-        <v>35</v>
-      </c>
+      <c r="A15" s="18"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="18" t="s">
+      <c r="A16" s="19" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="18" t="s">
         <v>37</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="18" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="18" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Label 16GB and 32GB prices as single sticks, not kits
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BFknSiXKDWdHdxsn9XQpko
</commit_message>
<xml_diff>
--- a/ram_bulk_pricing.xlsx
+++ b/ram_bulk_pricing.xlsx
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="43">
   <si>
     <t xml:space="preserve">RAM Bulk Buyer Pricing (all brands, non-gaming)</t>
   </si>
@@ -111,6 +111,12 @@
     <t xml:space="preserve">DDR4-2133 / PC4-17000</t>
   </si>
   <si>
+    <t xml:space="preserve">Single 16GB stick (not a kit)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Single 32GB stick (not a kit)</t>
+  </si>
+  <si>
     <t xml:space="preserve">DDR4-2400 / PC4-19200</t>
   </si>
   <si>
@@ -138,7 +144,10 @@
     <t xml:space="preserve">8GB and up: desktop and laptop are the same price; server is priced separately.</t>
   </si>
   <si>
-    <t xml:space="preserve">DDR4 16GB = 2 x the 8GB price + $2.50.  DDR4 32GB = 2 x the 16GB price + $2.50.  DDR3 16/32GB not priced.</t>
+    <t xml:space="preserve">All prices are for ONE stick. 16GB and 32GB rows are single 16GB / 32GB sticks, not kits.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DDR4 16GB stick = 2 x the 8GB price + $2.50.  DDR4 32GB stick = 2 x the 16GB price + $2.50.  DDR3 16/32GB not priced.</t>
   </si>
   <si>
     <t xml:space="preserve">Rows are grouped by speed; the shading alternates between speed groups.</t>
@@ -1295,7 +1304,9 @@
         <f aca="false">IF(OR(E23="",G23=""),"",E23*G23)</f>
         <v/>
       </c>
-      <c r="I23" s="12"/>
+      <c r="I23" s="12" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
@@ -1322,7 +1333,9 @@
         <f aca="false">IF(OR(E24="",G24=""),"",E24*G24)</f>
         <v/>
       </c>
-      <c r="I24" s="12"/>
+      <c r="I24" s="12" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
@@ -1374,7 +1387,9 @@
         <f aca="false">IF(OR(E26="",G26=""),"",E26*G26)</f>
         <v/>
       </c>
-      <c r="I26" s="12"/>
+      <c r="I26" s="12" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
@@ -1401,7 +1416,9 @@
         <f aca="false">IF(OR(E27="",G27=""),"",E27*G27)</f>
         <v/>
       </c>
-      <c r="I27" s="12"/>
+      <c r="I27" s="12" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
@@ -1433,7 +1450,7 @@
         <v>19</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C29" s="15" t="n">
         <v>4</v>
@@ -1460,7 +1477,7 @@
         <v>19</v>
       </c>
       <c r="B30" s="14" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C30" s="15" t="n">
         <v>4</v>
@@ -1487,7 +1504,7 @@
         <v>19</v>
       </c>
       <c r="B31" s="14" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C31" s="15" t="n">
         <v>4</v>
@@ -1514,7 +1531,7 @@
         <v>19</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C32" s="15" t="n">
         <v>8</v>
@@ -1541,7 +1558,7 @@
         <v>19</v>
       </c>
       <c r="B33" s="14" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C33" s="15" t="n">
         <v>8</v>
@@ -1568,7 +1585,7 @@
         <v>19</v>
       </c>
       <c r="B34" s="14" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C34" s="15" t="n">
         <v>8</v>
@@ -1593,7 +1610,7 @@
         <v>19</v>
       </c>
       <c r="B35" s="14" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C35" s="15" t="n">
         <v>16</v>
@@ -1613,14 +1630,16 @@
         <f aca="false">IF(OR(E35="",G35=""),"",E35*G35)</f>
         <v/>
       </c>
-      <c r="I35" s="12"/>
+      <c r="I35" s="12" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13" t="s">
         <v>19</v>
       </c>
       <c r="B36" s="14" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C36" s="15" t="n">
         <v>16</v>
@@ -1640,14 +1659,16 @@
         <f aca="false">IF(OR(E36="",G36=""),"",E36*G36)</f>
         <v/>
       </c>
-      <c r="I36" s="12"/>
+      <c r="I36" s="12" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13" t="s">
         <v>19</v>
       </c>
       <c r="B37" s="14" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C37" s="15" t="n">
         <v>16</v>
@@ -1672,7 +1693,7 @@
         <v>19</v>
       </c>
       <c r="B38" s="14" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C38" s="15" t="n">
         <v>32</v>
@@ -1692,14 +1713,16 @@
         <f aca="false">IF(OR(E38="",G38=""),"",E38*G38)</f>
         <v/>
       </c>
-      <c r="I38" s="12"/>
+      <c r="I38" s="12" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="13" t="s">
         <v>19</v>
       </c>
       <c r="B39" s="14" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C39" s="15" t="n">
         <v>32</v>
@@ -1719,14 +1742,16 @@
         <f aca="false">IF(OR(E39="",G39=""),"",E39*G39)</f>
         <v/>
       </c>
-      <c r="I39" s="12"/>
+      <c r="I39" s="12" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="13" t="s">
         <v>19</v>
       </c>
       <c r="B40" s="14" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C40" s="15" t="n">
         <v>32</v>
@@ -1751,7 +1776,7 @@
         <v>19</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C41" s="9" t="n">
         <v>4</v>
@@ -1778,7 +1803,7 @@
         <v>19</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C42" s="9" t="n">
         <v>4</v>
@@ -1805,7 +1830,7 @@
         <v>19</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C43" s="9" t="n">
         <v>4</v>
@@ -1832,7 +1857,7 @@
         <v>19</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C44" s="9" t="n">
         <v>8</v>
@@ -1859,7 +1884,7 @@
         <v>19</v>
       </c>
       <c r="B45" s="8" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C45" s="9" t="n">
         <v>8</v>
@@ -1886,7 +1911,7 @@
         <v>19</v>
       </c>
       <c r="B46" s="8" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C46" s="9" t="n">
         <v>8</v>
@@ -1911,7 +1936,7 @@
         <v>19</v>
       </c>
       <c r="B47" s="8" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C47" s="9" t="n">
         <v>16</v>
@@ -1931,14 +1956,16 @@
         <f aca="false">IF(OR(E47="",G47=""),"",E47*G47)</f>
         <v/>
       </c>
-      <c r="I47" s="12"/>
+      <c r="I47" s="12" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="s">
         <v>19</v>
       </c>
       <c r="B48" s="8" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C48" s="9" t="n">
         <v>16</v>
@@ -1958,14 +1985,16 @@
         <f aca="false">IF(OR(E48="",G48=""),"",E48*G48)</f>
         <v/>
       </c>
-      <c r="I48" s="12"/>
+      <c r="I48" s="12" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="7" t="s">
         <v>19</v>
       </c>
       <c r="B49" s="8" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C49" s="9" t="n">
         <v>16</v>
@@ -1990,7 +2019,7 @@
         <v>19</v>
       </c>
       <c r="B50" s="8" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C50" s="9" t="n">
         <v>32</v>
@@ -2010,14 +2039,16 @@
         <f aca="false">IF(OR(E50="",G50=""),"",E50*G50)</f>
         <v/>
       </c>
-      <c r="I50" s="12"/>
+      <c r="I50" s="12" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="7" t="s">
         <v>19</v>
       </c>
       <c r="B51" s="8" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C51" s="9" t="n">
         <v>32</v>
@@ -2037,14 +2068,16 @@
         <f aca="false">IF(OR(E51="",G51=""),"",E51*G51)</f>
         <v/>
       </c>
-      <c r="I51" s="12"/>
+      <c r="I51" s="12" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="s">
         <v>19</v>
       </c>
       <c r="B52" s="8" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C52" s="9" t="n">
         <v>32</v>
@@ -2069,7 +2102,7 @@
         <v>19</v>
       </c>
       <c r="B53" s="14" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C53" s="15" t="n">
         <v>4</v>
@@ -2096,7 +2129,7 @@
         <v>19</v>
       </c>
       <c r="B54" s="14" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C54" s="15" t="n">
         <v>4</v>
@@ -2123,7 +2156,7 @@
         <v>19</v>
       </c>
       <c r="B55" s="14" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C55" s="15" t="n">
         <v>4</v>
@@ -2150,7 +2183,7 @@
         <v>19</v>
       </c>
       <c r="B56" s="14" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C56" s="15" t="n">
         <v>8</v>
@@ -2177,7 +2210,7 @@
         <v>19</v>
       </c>
       <c r="B57" s="14" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C57" s="15" t="n">
         <v>8</v>
@@ -2204,7 +2237,7 @@
         <v>19</v>
       </c>
       <c r="B58" s="14" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C58" s="15" t="n">
         <v>8</v>
@@ -2229,7 +2262,7 @@
         <v>19</v>
       </c>
       <c r="B59" s="14" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C59" s="15" t="n">
         <v>16</v>
@@ -2249,14 +2282,16 @@
         <f aca="false">IF(OR(E59="",G59=""),"",E59*G59)</f>
         <v/>
       </c>
-      <c r="I59" s="12"/>
+      <c r="I59" s="12" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="13" t="s">
         <v>19</v>
       </c>
       <c r="B60" s="14" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C60" s="15" t="n">
         <v>16</v>
@@ -2276,14 +2311,16 @@
         <f aca="false">IF(OR(E60="",G60=""),"",E60*G60)</f>
         <v/>
       </c>
-      <c r="I60" s="12"/>
+      <c r="I60" s="12" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="13" t="s">
         <v>19</v>
       </c>
       <c r="B61" s="14" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C61" s="15" t="n">
         <v>16</v>
@@ -2308,7 +2345,7 @@
         <v>19</v>
       </c>
       <c r="B62" s="14" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C62" s="15" t="n">
         <v>32</v>
@@ -2328,14 +2365,16 @@
         <f aca="false">IF(OR(E62="",G62=""),"",E62*G62)</f>
         <v/>
       </c>
-      <c r="I62" s="12"/>
+      <c r="I62" s="12" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="13" t="s">
         <v>19</v>
       </c>
       <c r="B63" s="14" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C63" s="15" t="n">
         <v>32</v>
@@ -2355,14 +2394,16 @@
         <f aca="false">IF(OR(E63="",G63=""),"",E63*G63)</f>
         <v/>
       </c>
-      <c r="I63" s="12"/>
+      <c r="I63" s="12" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="13" t="s">
         <v>19</v>
       </c>
       <c r="B64" s="14" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C64" s="15" t="n">
         <v>32</v>
@@ -2407,7 +2448,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="110"/>
@@ -2415,7 +2456,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="17" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2423,83 +2464,88 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="18" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="18"/>
+      <c r="A10" s="18" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19" t="s">
-        <v>32</v>
-      </c>
+      <c r="A11" s="18"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="18" t="s">
-        <v>33</v>
+      <c r="A12" s="19" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="18"/>
+      <c r="A15" s="18" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="19" t="s">
-        <v>36</v>
-      </c>
+      <c r="A16" s="18"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="18" t="s">
-        <v>37</v>
+      <c r="A17" s="19" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="18" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="18" t="s">
-        <v>39</v>
+        <v>41</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="18" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Price 8GB DDR4-2133/2400 server RDIMMs at $20
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BFknSiXKDWdHdxsn9XQpko
</commit_message>
<xml_diff>
--- a/ram_bulk_pricing.xlsx
+++ b/ram_bulk_pricing.xlsx
@@ -1267,10 +1267,12 @@
       <c r="D22" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="E22" s="10"/>
-      <c r="F22" s="11" t="str">
+      <c r="E22" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="F22" s="11" t="n">
         <f aca="false">IF(E22="","",E22/C22)</f>
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="G22" s="12"/>
       <c r="H22" s="11" t="str">
@@ -1593,10 +1595,12 @@
       <c r="D34" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="E34" s="10"/>
-      <c r="F34" s="16" t="str">
+      <c r="E34" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="F34" s="16" t="n">
         <f aca="false">IF(E34="","",E34/C34)</f>
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="G34" s="12"/>
       <c r="H34" s="16" t="str">

</xml_diff>

<commit_message>
Price 16GB and 32GB DDR4-2133 server RDIMMs
16GB = 2x8GB + $2.50 ($42.50), 32GB = 2x16GB + $2.50 ($87.50).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BFknSiXKDWdHdxsn9XQpko
</commit_message>
<xml_diff>
--- a/ram_bulk_pricing.xlsx
+++ b/ram_bulk_pricing.xlsx
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="44">
   <si>
     <t xml:space="preserve">RAM Bulk Buyer Pricing (all brands, non-gaming)</t>
   </si>
@@ -142,6 +142,9 @@
   </si>
   <si>
     <t xml:space="preserve">8GB and up: desktop and laptop are the same price; server is priced separately.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Server DDR4-2133: 16GB stick = 2 x the 8GB server price + $2.50; 32GB = 2 x the 16GB server price + $2.50.</t>
   </si>
   <si>
     <t xml:space="preserve">All prices are for ONE stick. 16GB and 32GB rows are single 16GB / 32GB sticks, not kits.</t>
@@ -1352,17 +1355,21 @@
       <c r="D25" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="E25" s="10"/>
-      <c r="F25" s="11" t="str">
+      <c r="E25" s="10" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="F25" s="11" t="n">
         <f aca="false">IF(E25="","",E25/C25)</f>
-        <v/>
+        <v>2.65625</v>
       </c>
       <c r="G25" s="12"/>
       <c r="H25" s="11" t="str">
         <f aca="false">IF(OR(E25="",G25=""),"",E25*G25)</f>
         <v/>
       </c>
-      <c r="I25" s="12"/>
+      <c r="I25" s="12" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
@@ -1435,17 +1442,21 @@
       <c r="D28" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="E28" s="10"/>
-      <c r="F28" s="11" t="str">
+      <c r="E28" s="10" t="n">
+        <v>87.5</v>
+      </c>
+      <c r="F28" s="11" t="n">
         <f aca="false">IF(E28="","",E28/C28)</f>
-        <v/>
+        <v>2.734375</v>
       </c>
       <c r="G28" s="12"/>
       <c r="H28" s="11" t="str">
         <f aca="false">IF(OR(E28="",G28=""),"",E28*G28)</f>
         <v/>
       </c>
-      <c r="I28" s="12"/>
+      <c r="I28" s="12" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="13" t="s">
@@ -2452,7 +2463,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="110"/>
@@ -2507,15 +2518,15 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="18"/>
+      <c r="A11" s="18" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="19" t="s">
-        <v>35</v>
-      </c>
+      <c r="A12" s="18"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="18" t="s">
+      <c r="A13" s="19" t="s">
         <v>36</v>
       </c>
     </row>
@@ -2530,15 +2541,15 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="18"/>
+      <c r="A16" s="18" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="19" t="s">
-        <v>39</v>
-      </c>
+      <c r="A17" s="18"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="18" t="s">
+      <c r="A18" s="19" t="s">
         <v>40</v>
       </c>
     </row>
@@ -2550,6 +2561,11 @@
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="18" t="s">
         <v>42</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="18" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Match remaining server prices to desktop/laptop
Keeps owner-set server prices for 8GB DDR4-2133/2400 and DDR4-2133 16/32GB.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BFknSiXKDWdHdxsn9XQpko
</commit_message>
<xml_diff>
--- a/ram_bulk_pricing.xlsx
+++ b/ram_bulk_pricing.xlsx
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="44">
   <si>
     <t xml:space="preserve">RAM Bulk Buyer Pricing (all brands, non-gaming)</t>
   </si>
@@ -141,7 +141,7 @@
     <t xml:space="preserve">4GB: desktop, laptop and server are all the same price for a given speed.</t>
   </si>
   <si>
-    <t xml:space="preserve">8GB and up: desktop and laptop are the same price; server is priced separately.</t>
+    <t xml:space="preserve">Server matches desktop/laptop prices, except 8GB DDR4-2133/2400 server ($20) and DDR4-2133 16/32GB server below.</t>
   </si>
   <si>
     <t xml:space="preserve">Server DDR4-2133: 16GB stick = 2 x the 8GB server price + $2.50; 32GB = 2 x the 16GB server price + $2.50.</t>
@@ -950,10 +950,12 @@
       <c r="D10" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="E10" s="10"/>
-      <c r="F10" s="11" t="str">
+      <c r="E10" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="F10" s="11" t="n">
         <f aca="false">IF(E10="","",E10/C10)</f>
-        <v/>
+        <v>1.375</v>
       </c>
       <c r="G10" s="12"/>
       <c r="H10" s="11" t="str">
@@ -1110,10 +1112,12 @@
       <c r="D16" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="E16" s="10"/>
-      <c r="F16" s="16" t="str">
+      <c r="E16" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="F16" s="16" t="n">
         <f aca="false">IF(E16="","",E16/C16)</f>
-        <v/>
+        <v>1.375</v>
       </c>
       <c r="G16" s="12"/>
       <c r="H16" s="16" t="str">
@@ -1691,17 +1695,21 @@
       <c r="D37" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="E37" s="10"/>
-      <c r="F37" s="16" t="str">
+      <c r="E37" s="10" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="F37" s="16" t="n">
         <f aca="false">IF(E37="","",E37/C37)</f>
-        <v/>
+        <v>2.90625</v>
       </c>
       <c r="G37" s="12"/>
       <c r="H37" s="16" t="str">
         <f aca="false">IF(OR(E37="",G37=""),"",E37*G37)</f>
         <v/>
       </c>
-      <c r="I37" s="12"/>
+      <c r="I37" s="12" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="13" t="s">
@@ -1774,17 +1782,21 @@
       <c r="D40" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="E40" s="10"/>
-      <c r="F40" s="16" t="str">
+      <c r="E40" s="10" t="n">
+        <v>95.5</v>
+      </c>
+      <c r="F40" s="16" t="n">
         <f aca="false">IF(E40="","",E40/C40)</f>
-        <v/>
+        <v>2.984375</v>
       </c>
       <c r="G40" s="12"/>
       <c r="H40" s="16" t="str">
         <f aca="false">IF(OR(E40="",G40=""),"",E40*G40)</f>
         <v/>
       </c>
-      <c r="I40" s="12"/>
+      <c r="I40" s="12" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
@@ -1934,10 +1946,12 @@
       <c r="D46" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="E46" s="10"/>
-      <c r="F46" s="11" t="str">
+      <c r="E46" s="10" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="F46" s="11" t="n">
         <f aca="false">IF(E46="","",E46/C46)</f>
-        <v/>
+        <v>2.9375</v>
       </c>
       <c r="G46" s="12"/>
       <c r="H46" s="11" t="str">
@@ -2017,17 +2031,21 @@
       <c r="D49" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="E49" s="10"/>
-      <c r="F49" s="11" t="str">
+      <c r="E49" s="10" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="F49" s="11" t="n">
         <f aca="false">IF(E49="","",E49/C49)</f>
-        <v/>
+        <v>3.09375</v>
       </c>
       <c r="G49" s="12"/>
       <c r="H49" s="11" t="str">
         <f aca="false">IF(OR(E49="",G49=""),"",E49*G49)</f>
         <v/>
       </c>
-      <c r="I49" s="12"/>
+      <c r="I49" s="12" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="s">
@@ -2100,17 +2118,21 @@
       <c r="D52" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="E52" s="10"/>
-      <c r="F52" s="11" t="str">
+      <c r="E52" s="10" t="n">
+        <v>101.5</v>
+      </c>
+      <c r="F52" s="11" t="n">
         <f aca="false">IF(E52="","",E52/C52)</f>
-        <v/>
+        <v>3.171875</v>
       </c>
       <c r="G52" s="12"/>
       <c r="H52" s="11" t="str">
         <f aca="false">IF(OR(E52="",G52=""),"",E52*G52)</f>
         <v/>
       </c>
-      <c r="I52" s="12"/>
+      <c r="I52" s="12" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="13" t="s">
@@ -2260,10 +2282,12 @@
       <c r="D58" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="E58" s="10"/>
-      <c r="F58" s="16" t="str">
+      <c r="E58" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="F58" s="16" t="n">
         <f aca="false">IF(E58="","",E58/C58)</f>
-        <v/>
+        <v>3.125</v>
       </c>
       <c r="G58" s="12"/>
       <c r="H58" s="16" t="str">
@@ -2343,17 +2367,21 @@
       <c r="D61" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="E61" s="10"/>
-      <c r="F61" s="16" t="str">
+      <c r="E61" s="10" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="F61" s="16" t="n">
         <f aca="false">IF(E61="","",E61/C61)</f>
-        <v/>
+        <v>3.28125</v>
       </c>
       <c r="G61" s="12"/>
       <c r="H61" s="16" t="str">
         <f aca="false">IF(OR(E61="",G61=""),"",E61*G61)</f>
         <v/>
       </c>
-      <c r="I61" s="12"/>
+      <c r="I61" s="12" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="13" t="s">
@@ -2426,17 +2454,21 @@
       <c r="D64" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="E64" s="10"/>
-      <c r="F64" s="16" t="str">
+      <c r="E64" s="10" t="n">
+        <v>107.5</v>
+      </c>
+      <c r="F64" s="16" t="n">
         <f aca="false">IF(E64="","",E64/C64)</f>
-        <v/>
+        <v>3.359375</v>
       </c>
       <c r="G64" s="12"/>
       <c r="H64" s="16" t="str">
         <f aca="false">IF(OR(E64="",G64=""),"",E64*G64)</f>
         <v/>
       </c>
-      <c r="I64" s="12"/>
+      <c r="I64" s="12" t="s">
+        <v>22</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:I64"/>

</xml_diff>

<commit_message>
Add eBay DDR3 bulk lot listing and lot sheet
Transcribed from owner's handwritten list; prices pulled from the
Bulk Pricing tab. 71 sticks, $589.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BFknSiXKDWdHdxsn9XQpko
</commit_message>
<xml_diff>
--- a/ram_bulk_pricing.xlsx
+++ b/ram_bulk_pricing.xlsx
@@ -10,6 +10,7 @@
   <sheets>
     <sheet name="Bulk Pricing" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="How to use" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="eBay Bulk Lot" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Bulk Pricing'!$A$4:$I$64</definedName>
@@ -46,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="60">
   <si>
     <t xml:space="preserve">RAM Bulk Buyer Pricing (all brands, non-gaming)</t>
   </si>
@@ -178,6 +179,54 @@
   </si>
   <si>
     <t xml:space="preserve">DDR4-2666 = PC4-21300 (2666V)   DDR4-3200 = PC4-25600 (3200AA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">eBay Bulk Lot - DDR3 (all tested)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lot total:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delete a row to remove an item; totals update. Price comes from the Bulk Pricing tab.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Line</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brand</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Line total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Samsung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADATA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G.Skill</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kingston</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Micron</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SK Hynix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nanya</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ramaxel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TeamGroup</t>
   </si>
 </sst>
 </file>
@@ -190,7 +239,7 @@
     <numFmt numFmtId="166" formatCode="\$#,##0.00"/>
     <numFmt numFmtId="167" formatCode="0&quot;GB&quot;"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -266,6 +315,21 @@
       <b val="true"/>
       <sz val="11"/>
       <color rgb="FF1F4E78"/>
+      <name val="Calibri"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i val="true"/>
+      <sz val="11"/>
+      <color rgb="FF595959"/>
+      <name val="Calibri"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF008000"/>
       <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
@@ -346,7 +410,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="25">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -424,6 +488,26 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -533,7 +617,7 @@
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF595959"/>
       <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF339966"/>
@@ -2609,4 +2693,865 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:M27"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <f aca="false">SUM(F5:F1000)</f>
+        <v>71</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D2" s="5" t="n">
+        <f aca="false">SUM(H5:H1000)</f>
+        <v>589</v>
+      </c>
+      <c r="E2" s="20" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="K4" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="L4" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="M4" s="21" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" s="23" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C5,'Bulk Pricing'!$C:$C,D5,'Bulk Pricing'!$D:$D,E5)</f>
+        <v>7</v>
+      </c>
+      <c r="H5" s="11" t="n">
+        <f aca="false">IF(F5="","",F5*G5)</f>
+        <v>14</v>
+      </c>
+      <c r="I5" s="8"/>
+      <c r="K5" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="L5" s="7" t="n">
+        <f aca="false">SUMIFS($F$5:$F$1000,$B$5:$B$1000,K5)</f>
+        <v>1</v>
+      </c>
+      <c r="M5" s="11" t="n">
+        <f aca="false">SUMIFS($H$5:$H$1000,$B$5:$B$1000,K5)</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>9</v>
+      </c>
+      <c r="G6" s="23" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C6,'Bulk Pricing'!$C:$C,D6,'Bulk Pricing'!$D:$D,E6)</f>
+        <v>7</v>
+      </c>
+      <c r="H6" s="11" t="n">
+        <f aca="false">IF(F6="","",F6*G6)</f>
+        <v>63</v>
+      </c>
+      <c r="I6" s="8"/>
+      <c r="K6" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="L6" s="7" t="n">
+        <f aca="false">SUMIFS($F$5:$F$1000,$B$5:$B$1000,K6)</f>
+        <v>2</v>
+      </c>
+      <c r="M6" s="11" t="n">
+        <f aca="false">SUMIFS($H$5:$H$1000,$B$5:$B$1000,K6)</f>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F7" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G7" s="23" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C7,'Bulk Pricing'!$C:$C,D7,'Bulk Pricing'!$D:$D,E7)</f>
+        <v>7</v>
+      </c>
+      <c r="H7" s="11" t="n">
+        <f aca="false">IF(F7="","",F7*G7)</f>
+        <v>14</v>
+      </c>
+      <c r="I7" s="8"/>
+      <c r="K7" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="L7" s="7" t="n">
+        <f aca="false">SUMIFS($F$5:$F$1000,$B$5:$B$1000,K7)</f>
+        <v>12</v>
+      </c>
+      <c r="M7" s="11" t="n">
+        <f aca="false">SUMIFS($H$5:$H$1000,$B$5:$B$1000,K7)</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" s="23" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C8,'Bulk Pricing'!$C:$C,D8,'Bulk Pricing'!$D:$D,E8)</f>
+        <v>11</v>
+      </c>
+      <c r="H8" s="11" t="n">
+        <f aca="false">IF(F8="","",F8*G8)</f>
+        <v>22</v>
+      </c>
+      <c r="I8" s="8"/>
+      <c r="K8" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="L8" s="7" t="n">
+        <f aca="false">SUMIFS($F$5:$F$1000,$B$5:$B$1000,K8)</f>
+        <v>2</v>
+      </c>
+      <c r="M8" s="11" t="n">
+        <f aca="false">SUMIFS($H$5:$H$1000,$B$5:$B$1000,K8)</f>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G9" s="23" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C9,'Bulk Pricing'!$C:$C,D9,'Bulk Pricing'!$D:$D,E9)</f>
+        <v>7</v>
+      </c>
+      <c r="H9" s="11" t="n">
+        <f aca="false">IF(F9="","",F9*G9)</f>
+        <v>14</v>
+      </c>
+      <c r="I9" s="8"/>
+      <c r="K9" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="L9" s="7" t="n">
+        <f aca="false">SUMIFS($F$5:$F$1000,$B$5:$B$1000,K9)</f>
+        <v>2</v>
+      </c>
+      <c r="M9" s="11" t="n">
+        <f aca="false">SUMIFS($H$5:$H$1000,$B$5:$B$1000,K9)</f>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G10" s="23" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C10,'Bulk Pricing'!$C:$C,D10,'Bulk Pricing'!$D:$D,E10)</f>
+        <v>11</v>
+      </c>
+      <c r="H10" s="11" t="n">
+        <f aca="false">IF(F10="","",F10*G10)</f>
+        <v>22</v>
+      </c>
+      <c r="I10" s="8"/>
+      <c r="K10" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="L10" s="7" t="n">
+        <f aca="false">SUMIFS($F$5:$F$1000,$B$5:$B$1000,K10)</f>
+        <v>3</v>
+      </c>
+      <c r="M10" s="11" t="n">
+        <f aca="false">SUMIFS($H$5:$H$1000,$B$5:$B$1000,K10)</f>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F11" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="23" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C11,'Bulk Pricing'!$C:$C,D11,'Bulk Pricing'!$D:$D,E11)</f>
+        <v>7</v>
+      </c>
+      <c r="H11" s="11" t="n">
+        <f aca="false">IF(F11="","",F11*G11)</f>
+        <v>7</v>
+      </c>
+      <c r="I11" s="8"/>
+      <c r="K11" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="L11" s="7" t="n">
+        <f aca="false">SUMIFS($F$5:$F$1000,$B$5:$B$1000,K11)</f>
+        <v>29</v>
+      </c>
+      <c r="M11" s="11" t="n">
+        <f aca="false">SUMIFS($H$5:$H$1000,$B$5:$B$1000,K11)</f>
+        <v>223</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F12" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="G12" s="23" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C12,'Bulk Pricing'!$C:$C,D12,'Bulk Pricing'!$D:$D,E12)</f>
+        <v>7</v>
+      </c>
+      <c r="H12" s="11" t="n">
+        <f aca="false">IF(F12="","",F12*G12)</f>
+        <v>21</v>
+      </c>
+      <c r="I12" s="8"/>
+      <c r="K12" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="L12" s="7" t="n">
+        <f aca="false">SUMIFS($F$5:$F$1000,$B$5:$B$1000,K12)</f>
+        <v>18</v>
+      </c>
+      <c r="M12" s="11" t="n">
+        <f aca="false">SUMIFS($H$5:$H$1000,$B$5:$B$1000,K12)</f>
+        <v>150</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="C13" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="D13" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="E13" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="F13" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G13" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C13,'Bulk Pricing'!$C:$C,D13,'Bulk Pricing'!$D:$D,E13)</f>
+        <v>11</v>
+      </c>
+      <c r="H13" s="16" t="n">
+        <f aca="false">IF(F13="","",F13*G13)</f>
+        <v>22</v>
+      </c>
+      <c r="I13" s="14"/>
+      <c r="K13" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="L13" s="7" t="n">
+        <f aca="false">SUMIFS($F$5:$F$1000,$B$5:$B$1000,K13)</f>
+        <v>2</v>
+      </c>
+      <c r="M13" s="11" t="n">
+        <f aca="false">SUMIFS($H$5:$H$1000,$B$5:$B$1000,K13)</f>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="E14" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="F14" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="G14" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C14,'Bulk Pricing'!$C:$C,D14,'Bulk Pricing'!$D:$D,E14)</f>
+        <v>11</v>
+      </c>
+      <c r="H14" s="16" t="n">
+        <f aca="false">IF(F14="","",F14*G14)</f>
+        <v>44</v>
+      </c>
+      <c r="I14" s="14"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="13" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="C15" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="D15" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="E15" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="F15" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G15" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C15,'Bulk Pricing'!$C:$C,D15,'Bulk Pricing'!$D:$D,E15)</f>
+        <v>11</v>
+      </c>
+      <c r="H15" s="16" t="n">
+        <f aca="false">IF(F15="","",F15*G15)</f>
+        <v>22</v>
+      </c>
+      <c r="I15" s="14"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="D16" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E16" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="F16" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C16,'Bulk Pricing'!$C:$C,D16,'Bulk Pricing'!$D:$D,E16)</f>
+        <v>7</v>
+      </c>
+      <c r="H16" s="16" t="n">
+        <f aca="false">IF(F16="","",F16*G16)</f>
+        <v>7</v>
+      </c>
+      <c r="I16" s="14"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="13" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="C17" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="D17" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E17" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="F17" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="G17" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C17,'Bulk Pricing'!$C:$C,D17,'Bulk Pricing'!$D:$D,E17)</f>
+        <v>7</v>
+      </c>
+      <c r="H17" s="16" t="n">
+        <f aca="false">IF(F17="","",F17*G17)</f>
+        <v>21</v>
+      </c>
+      <c r="I17" s="14"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="13" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C18" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E18" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="F18" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G18" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C18,'Bulk Pricing'!$C:$C,D18,'Bulk Pricing'!$D:$D,E18)</f>
+        <v>7</v>
+      </c>
+      <c r="H18" s="16" t="n">
+        <f aca="false">IF(F18="","",F18*G18)</f>
+        <v>14</v>
+      </c>
+      <c r="I18" s="14"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C19" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E19" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F19" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="G19" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C19,'Bulk Pricing'!$C:$C,D19,'Bulk Pricing'!$D:$D,E19)</f>
+        <v>7</v>
+      </c>
+      <c r="H19" s="16" t="n">
+        <f aca="false">IF(F19="","",F19*G19)</f>
+        <v>35</v>
+      </c>
+      <c r="I19" s="14"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="13" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="C20" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="D20" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="E20" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F20" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G20" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C20,'Bulk Pricing'!$C:$C,D20,'Bulk Pricing'!$D:$D,E20)</f>
+        <v>11</v>
+      </c>
+      <c r="H20" s="16" t="n">
+        <f aca="false">IF(F20="","",F20*G20)</f>
+        <v>22</v>
+      </c>
+      <c r="I20" s="14"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C21" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="D21" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E21" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F21" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G21" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C21,'Bulk Pricing'!$C:$C,D21,'Bulk Pricing'!$D:$D,E21)</f>
+        <v>7</v>
+      </c>
+      <c r="H21" s="16" t="n">
+        <f aca="false">IF(F21="","",F21*G21)</f>
+        <v>14</v>
+      </c>
+      <c r="I21" s="14"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="13" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="C22" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="D22" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="E22" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F22" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G22" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C22,'Bulk Pricing'!$C:$C,D22,'Bulk Pricing'!$D:$D,E22)</f>
+        <v>11</v>
+      </c>
+      <c r="H22" s="16" t="n">
+        <f aca="false">IF(F22="","",F22*G22)</f>
+        <v>22</v>
+      </c>
+      <c r="I22" s="14"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="13" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="C23" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="D23" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="E23" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F23" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C23,'Bulk Pricing'!$C:$C,D23,'Bulk Pricing'!$D:$D,E23)</f>
+        <v>11</v>
+      </c>
+      <c r="H23" s="16" t="n">
+        <f aca="false">IF(F23="","",F23*G23)</f>
+        <v>11</v>
+      </c>
+      <c r="I23" s="14"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C24" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="D24" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="E24" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F24" s="22" t="n">
+        <v>6</v>
+      </c>
+      <c r="G24" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C24,'Bulk Pricing'!$C:$C,D24,'Bulk Pricing'!$D:$D,E24)</f>
+        <v>11</v>
+      </c>
+      <c r="H24" s="16" t="n">
+        <f aca="false">IF(F24="","",F24*G24)</f>
+        <v>66</v>
+      </c>
+      <c r="I24" s="14"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="13" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="C25" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="D25" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E25" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F25" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G25" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C25,'Bulk Pricing'!$C:$C,D25,'Bulk Pricing'!$D:$D,E25)</f>
+        <v>7</v>
+      </c>
+      <c r="H25" s="16" t="n">
+        <f aca="false">IF(F25="","",F25*G25)</f>
+        <v>70</v>
+      </c>
+      <c r="I25" s="14"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="13" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="C26" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="D26" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E26" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F26" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="G26" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C26,'Bulk Pricing'!$C:$C,D26,'Bulk Pricing'!$D:$D,E26)</f>
+        <v>7</v>
+      </c>
+      <c r="H26" s="16" t="n">
+        <f aca="false">IF(F26="","",F26*G26)</f>
+        <v>21</v>
+      </c>
+      <c r="I26" s="14"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="13" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="C27" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="D27" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E27" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F27" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="G27" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C27,'Bulk Pricing'!$C:$C,D27,'Bulk Pricing'!$D:$D,E27)</f>
+        <v>7</v>
+      </c>
+      <c r="H27" s="16" t="n">
+        <f aca="false">IF(F27="","",F27*G27)</f>
+        <v>21</v>
+      </c>
+      <c r="I27" s="14"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add eBay bulk lot 2 (DDR4) listing and lot sheet
107 sticks of DDR4-2133/2400, $1,967, from owner's handwritten list.
Lot sheets renamed to 'Lot 1 - DDR3' and 'Lot 2 - DDR4'.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BFknSiXKDWdHdxsn9XQpko
</commit_message>
<xml_diff>
--- a/ram_bulk_pricing.xlsx
+++ b/ram_bulk_pricing.xlsx
@@ -10,7 +10,8 @@
   <sheets>
     <sheet name="Bulk Pricing" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="How to use" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="eBay Bulk Lot" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Lot 1 - DDR3" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Lot 2 - DDR4" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Bulk Pricing'!$A$4:$I$64</definedName>
@@ -47,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="63">
   <si>
     <t xml:space="preserve">RAM Bulk Buyer Pricing (all brands, non-gaming)</t>
   </si>
@@ -181,7 +182,7 @@
     <t xml:space="preserve">DDR4-2666 = PC4-21300 (2666V)   DDR4-3200 = PC4-25600 (3200AA)</t>
   </si>
   <si>
-    <t xml:space="preserve">eBay Bulk Lot - DDR3 (all tested)</t>
+    <t xml:space="preserve">eBay Bulk Lot 1 - DDR3 (all tested)</t>
   </si>
   <si>
     <t xml:space="preserve">Lot total:</t>
@@ -227,6 +228,15 @@
   </si>
   <si>
     <t xml:space="preserve">TeamGroup</t>
+  </si>
+  <si>
+    <t xml:space="preserve">eBay Bulk Lot 2 - DDR4 (all tested)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Microtech</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crucial</t>
   </si>
 </sst>
 </file>
@@ -3554,4 +3564,785 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:M25"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <f aca="false">SUM(F5:F1000)</f>
+        <v>107</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D2" s="5" t="n">
+        <f aca="false">SUM(H5:H1000)</f>
+        <v>1967</v>
+      </c>
+      <c r="E2" s="20" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="K4" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="L4" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="M4" s="21" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>17</v>
+      </c>
+      <c r="G5" s="23" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C5,'Bulk Pricing'!$C:$C,D5,'Bulk Pricing'!$D:$D,E5)</f>
+        <v>11</v>
+      </c>
+      <c r="H5" s="11" t="n">
+        <f aca="false">IF(F5="","",F5*G5)</f>
+        <v>187</v>
+      </c>
+      <c r="I5" s="8"/>
+      <c r="K5" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="L5" s="7" t="n">
+        <f aca="false">SUMIFS($F$5:$F$1000,$B$5:$B$1000,K5)</f>
+        <v>2</v>
+      </c>
+      <c r="M5" s="11" t="n">
+        <f aca="false">SUMIFS($H$5:$H$1000,$B$5:$B$1000,K5)</f>
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="G6" s="23" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C6,'Bulk Pricing'!$C:$C,D6,'Bulk Pricing'!$D:$D,E6)</f>
+        <v>11</v>
+      </c>
+      <c r="H6" s="11" t="n">
+        <f aca="false">IF(F6="","",F6*G6)</f>
+        <v>44</v>
+      </c>
+      <c r="I6" s="8"/>
+      <c r="K6" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="L6" s="7" t="n">
+        <f aca="false">SUMIFS($F$5:$F$1000,$B$5:$B$1000,K6)</f>
+        <v>11</v>
+      </c>
+      <c r="M6" s="11" t="n">
+        <f aca="false">SUMIFS($H$5:$H$1000,$B$5:$B$1000,K6)</f>
+        <v>405</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F7" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="23" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C7,'Bulk Pricing'!$C:$C,D7,'Bulk Pricing'!$D:$D,E7)</f>
+        <v>11</v>
+      </c>
+      <c r="H7" s="11" t="n">
+        <f aca="false">IF(F7="","",F7*G7)</f>
+        <v>11</v>
+      </c>
+      <c r="I7" s="8"/>
+      <c r="K7" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="L7" s="7" t="n">
+        <f aca="false">SUMIFS($F$5:$F$1000,$B$5:$B$1000,K7)</f>
+        <v>5</v>
+      </c>
+      <c r="M7" s="11" t="n">
+        <f aca="false">SUMIFS($H$5:$H$1000,$B$5:$B$1000,K7)</f>
+        <v>88</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8" s="22" t="n">
+        <v>19</v>
+      </c>
+      <c r="G8" s="23" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C8,'Bulk Pricing'!$C:$C,D8,'Bulk Pricing'!$D:$D,E8)</f>
+        <v>22</v>
+      </c>
+      <c r="H8" s="11" t="n">
+        <f aca="false">IF(F8="","",F8*G8)</f>
+        <v>418</v>
+      </c>
+      <c r="I8" s="8"/>
+      <c r="K8" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="L8" s="7" t="n">
+        <f aca="false">SUMIFS($F$5:$F$1000,$B$5:$B$1000,K8)</f>
+        <v>37</v>
+      </c>
+      <c r="M8" s="11" t="n">
+        <f aca="false">SUMIFS($H$5:$H$1000,$B$5:$B$1000,K8)</f>
+        <v>627</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="23" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C9,'Bulk Pricing'!$C:$C,D9,'Bulk Pricing'!$D:$D,E9)</f>
+        <v>22</v>
+      </c>
+      <c r="H9" s="11" t="n">
+        <f aca="false">IF(F9="","",F9*G9)</f>
+        <v>22</v>
+      </c>
+      <c r="I9" s="8"/>
+      <c r="K9" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="L9" s="7" t="n">
+        <f aca="false">SUMIFS($F$5:$F$1000,$B$5:$B$1000,K9)</f>
+        <v>29</v>
+      </c>
+      <c r="M9" s="11" t="n">
+        <f aca="false">SUMIFS($H$5:$H$1000,$B$5:$B$1000,K9)</f>
+        <v>440</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G10" s="23" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C10,'Bulk Pricing'!$C:$C,D10,'Bulk Pricing'!$D:$D,E10)</f>
+        <v>22</v>
+      </c>
+      <c r="H10" s="11" t="n">
+        <f aca="false">IF(F10="","",F10*G10)</f>
+        <v>44</v>
+      </c>
+      <c r="I10" s="8"/>
+      <c r="K10" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="L10" s="7" t="n">
+        <f aca="false">SUMIFS($F$5:$F$1000,$B$5:$B$1000,K10)</f>
+        <v>21</v>
+      </c>
+      <c r="M10" s="11" t="n">
+        <f aca="false">SUMIFS($H$5:$H$1000,$B$5:$B$1000,K10)</f>
+        <v>319</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F11" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G11" s="23" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C11,'Bulk Pricing'!$C:$C,D11,'Bulk Pricing'!$D:$D,E11)</f>
+        <v>22</v>
+      </c>
+      <c r="H11" s="11" t="n">
+        <f aca="false">IF(F11="","",F11*G11)</f>
+        <v>44</v>
+      </c>
+      <c r="I11" s="8"/>
+      <c r="K11" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="L11" s="7" t="n">
+        <f aca="false">SUMIFS($F$5:$F$1000,$B$5:$B$1000,K11)</f>
+        <v>2</v>
+      </c>
+      <c r="M11" s="11" t="n">
+        <f aca="false">SUMIFS($H$5:$H$1000,$B$5:$B$1000,K11)</f>
+        <v>44</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F12" s="22" t="n">
+        <v>6</v>
+      </c>
+      <c r="G12" s="23" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C12,'Bulk Pricing'!$C:$C,D12,'Bulk Pricing'!$D:$D,E12)</f>
+        <v>11</v>
+      </c>
+      <c r="H12" s="11" t="n">
+        <f aca="false">IF(F12="","",F12*G12)</f>
+        <v>66</v>
+      </c>
+      <c r="I12" s="8"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="C13" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D13" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E13" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F13" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="G13" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C13,'Bulk Pricing'!$C:$C,D13,'Bulk Pricing'!$D:$D,E13)</f>
+        <v>11</v>
+      </c>
+      <c r="H13" s="16" t="n">
+        <f aca="false">IF(F13="","",F13*G13)</f>
+        <v>88</v>
+      </c>
+      <c r="I13" s="14"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D14" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="E14" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F14" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="G14" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C14,'Bulk Pricing'!$C:$C,D14,'Bulk Pricing'!$D:$D,E14)</f>
+        <v>46.5</v>
+      </c>
+      <c r="H14" s="16" t="n">
+        <f aca="false">IF(F14="","",F14*G14)</f>
+        <v>372</v>
+      </c>
+      <c r="I14" s="14"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="13" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="C15" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D15" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="E15" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F15" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="G15" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C15,'Bulk Pricing'!$C:$C,D15,'Bulk Pricing'!$D:$D,E15)</f>
+        <v>22</v>
+      </c>
+      <c r="H15" s="16" t="n">
+        <f aca="false">IF(F15="","",F15*G15)</f>
+        <v>176</v>
+      </c>
+      <c r="I15" s="14"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D16" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="E16" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F16" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="G16" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C16,'Bulk Pricing'!$C:$C,D16,'Bulk Pricing'!$D:$D,E16)</f>
+        <v>22</v>
+      </c>
+      <c r="H16" s="16" t="n">
+        <f aca="false">IF(F16="","",F16*G16)</f>
+        <v>176</v>
+      </c>
+      <c r="I16" s="14"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="13" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="C17" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D17" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="E17" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F17" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G17" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C17,'Bulk Pricing'!$C:$C,D17,'Bulk Pricing'!$D:$D,E17)</f>
+        <v>22</v>
+      </c>
+      <c r="H17" s="16" t="n">
+        <f aca="false">IF(F17="","",F17*G17)</f>
+        <v>44</v>
+      </c>
+      <c r="I17" s="14"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="13" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="C18" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D18" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E18" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F18" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G18" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C18,'Bulk Pricing'!$C:$C,D18,'Bulk Pricing'!$D:$D,E18)</f>
+        <v>11</v>
+      </c>
+      <c r="H18" s="16" t="n">
+        <f aca="false">IF(F18="","",F18*G18)</f>
+        <v>22</v>
+      </c>
+      <c r="I18" s="14"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C19" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D19" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E19" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F19" s="22" t="n">
+        <v>7</v>
+      </c>
+      <c r="G19" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C19,'Bulk Pricing'!$C:$C,D19,'Bulk Pricing'!$D:$D,E19)</f>
+        <v>11</v>
+      </c>
+      <c r="H19" s="16" t="n">
+        <f aca="false">IF(F19="","",F19*G19)</f>
+        <v>77</v>
+      </c>
+      <c r="I19" s="14"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="13" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="C20" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D20" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="E20" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F20" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="G20" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C20,'Bulk Pricing'!$C:$C,D20,'Bulk Pricing'!$D:$D,E20)</f>
+        <v>22</v>
+      </c>
+      <c r="H20" s="16" t="n">
+        <f aca="false">IF(F20="","",F20*G20)</f>
+        <v>66</v>
+      </c>
+      <c r="I20" s="14"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="C21" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D21" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E21" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="F21" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="G21" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C21,'Bulk Pricing'!$C:$C,D21,'Bulk Pricing'!$D:$D,E21)</f>
+        <v>11</v>
+      </c>
+      <c r="H21" s="16" t="n">
+        <f aca="false">IF(F21="","",F21*G21)</f>
+        <v>33</v>
+      </c>
+      <c r="I21" s="14"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="13" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="C22" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D22" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="E22" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="F22" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C22,'Bulk Pricing'!$C:$C,D22,'Bulk Pricing'!$D:$D,E22)</f>
+        <v>22</v>
+      </c>
+      <c r="H22" s="16" t="n">
+        <f aca="false">IF(F22="","",F22*G22)</f>
+        <v>22</v>
+      </c>
+      <c r="I22" s="14"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="13" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="C23" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D23" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E23" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="F23" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G23" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C23,'Bulk Pricing'!$C:$C,D23,'Bulk Pricing'!$D:$D,E23)</f>
+        <v>11</v>
+      </c>
+      <c r="H23" s="16" t="n">
+        <f aca="false">IF(F23="","",F23*G23)</f>
+        <v>22</v>
+      </c>
+      <c r="I23" s="14"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="C24" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D24" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E24" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="F24" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C24,'Bulk Pricing'!$C:$C,D24,'Bulk Pricing'!$D:$D,E24)</f>
+        <v>11</v>
+      </c>
+      <c r="H24" s="16" t="n">
+        <f aca="false">IF(F24="","",F24*G24)</f>
+        <v>11</v>
+      </c>
+      <c r="I24" s="14"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="13" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C25" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D25" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E25" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="F25" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G25" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C25,'Bulk Pricing'!$C:$C,D25,'Bulk Pricing'!$D:$D,E25)</f>
+        <v>11</v>
+      </c>
+      <c r="H25" s="16" t="n">
+        <f aca="false">IF(F25="","",F25*G25)</f>
+        <v>22</v>
+      </c>
+      <c r="I25" s="14"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add eBay bulk lots 3 (DDR4-2666/3200) and 4 (server + Cisco)
Lot 3: 56 desktop/laptop sticks, $1,408. Lot 4: 8x SK Hynix 32GB
DDR4-3200 RDIMM + 9x Cisco 4GB at $24.99, $1,084.91.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BFknSiXKDWdHdxsn9XQpko
</commit_message>
<xml_diff>
--- a/ram_bulk_pricing.xlsx
+++ b/ram_bulk_pricing.xlsx
@@ -12,6 +12,8 @@
     <sheet name="How to use" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Lot 1 - DDR3" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Lot 2 - DDR4" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Lot 3 - DDR4 2666-3200" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Lot 4 - Server &amp; Cisco" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Bulk Pricing'!$A$4:$I$64</definedName>
@@ -48,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="531" uniqueCount="68">
   <si>
     <t xml:space="preserve">RAM Bulk Buyer Pricing (all brands, non-gaming)</t>
   </si>
@@ -237,6 +239,21 @@
   </si>
   <si>
     <t xml:space="preserve">Crucial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">eBay Bulk Lot 3 - DDR4 2666/3200 (all tested)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forza</t>
+  </si>
+  <si>
+    <t xml:space="preserve">eBay Bulk Lot 4 - Server &amp; Cisco (all tested)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cisco</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cisco DRAM module</t>
   </si>
 </sst>
 </file>
@@ -2813,7 +2830,7 @@
         <v>7</v>
       </c>
       <c r="H5" s="11" t="n">
-        <f aca="false">IF(F5="","",F5*G5)</f>
+        <f aca="false">IF(OR(F5="",G5=""),"",F5*G5)</f>
         <v>14</v>
       </c>
       <c r="I5" s="8"/>
@@ -2853,7 +2870,7 @@
         <v>7</v>
       </c>
       <c r="H6" s="11" t="n">
-        <f aca="false">IF(F6="","",F6*G6)</f>
+        <f aca="false">IF(OR(F6="",G6=""),"",F6*G6)</f>
         <v>63</v>
       </c>
       <c r="I6" s="8"/>
@@ -2893,7 +2910,7 @@
         <v>7</v>
       </c>
       <c r="H7" s="11" t="n">
-        <f aca="false">IF(F7="","",F7*G7)</f>
+        <f aca="false">IF(OR(F7="",G7=""),"",F7*G7)</f>
         <v>14</v>
       </c>
       <c r="I7" s="8"/>
@@ -2933,7 +2950,7 @@
         <v>11</v>
       </c>
       <c r="H8" s="11" t="n">
-        <f aca="false">IF(F8="","",F8*G8)</f>
+        <f aca="false">IF(OR(F8="",G8=""),"",F8*G8)</f>
         <v>22</v>
       </c>
       <c r="I8" s="8"/>
@@ -2973,7 +2990,7 @@
         <v>7</v>
       </c>
       <c r="H9" s="11" t="n">
-        <f aca="false">IF(F9="","",F9*G9)</f>
+        <f aca="false">IF(OR(F9="",G9=""),"",F9*G9)</f>
         <v>14</v>
       </c>
       <c r="I9" s="8"/>
@@ -3013,7 +3030,7 @@
         <v>11</v>
       </c>
       <c r="H10" s="11" t="n">
-        <f aca="false">IF(F10="","",F10*G10)</f>
+        <f aca="false">IF(OR(F10="",G10=""),"",F10*G10)</f>
         <v>22</v>
       </c>
       <c r="I10" s="8"/>
@@ -3053,7 +3070,7 @@
         <v>7</v>
       </c>
       <c r="H11" s="11" t="n">
-        <f aca="false">IF(F11="","",F11*G11)</f>
+        <f aca="false">IF(OR(F11="",G11=""),"",F11*G11)</f>
         <v>7</v>
       </c>
       <c r="I11" s="8"/>
@@ -3093,7 +3110,7 @@
         <v>7</v>
       </c>
       <c r="H12" s="11" t="n">
-        <f aca="false">IF(F12="","",F12*G12)</f>
+        <f aca="false">IF(OR(F12="",G12=""),"",F12*G12)</f>
         <v>21</v>
       </c>
       <c r="I12" s="8"/>
@@ -3133,7 +3150,7 @@
         <v>11</v>
       </c>
       <c r="H13" s="16" t="n">
-        <f aca="false">IF(F13="","",F13*G13)</f>
+        <f aca="false">IF(OR(F13="",G13=""),"",F13*G13)</f>
         <v>22</v>
       </c>
       <c r="I13" s="14"/>
@@ -3173,7 +3190,7 @@
         <v>11</v>
       </c>
       <c r="H14" s="16" t="n">
-        <f aca="false">IF(F14="","",F14*G14)</f>
+        <f aca="false">IF(OR(F14="",G14=""),"",F14*G14)</f>
         <v>44</v>
       </c>
       <c r="I14" s="14"/>
@@ -3202,7 +3219,7 @@
         <v>11</v>
       </c>
       <c r="H15" s="16" t="n">
-        <f aca="false">IF(F15="","",F15*G15)</f>
+        <f aca="false">IF(OR(F15="",G15=""),"",F15*G15)</f>
         <v>22</v>
       </c>
       <c r="I15" s="14"/>
@@ -3231,7 +3248,7 @@
         <v>7</v>
       </c>
       <c r="H16" s="16" t="n">
-        <f aca="false">IF(F16="","",F16*G16)</f>
+        <f aca="false">IF(OR(F16="",G16=""),"",F16*G16)</f>
         <v>7</v>
       </c>
       <c r="I16" s="14"/>
@@ -3260,7 +3277,7 @@
         <v>7</v>
       </c>
       <c r="H17" s="16" t="n">
-        <f aca="false">IF(F17="","",F17*G17)</f>
+        <f aca="false">IF(OR(F17="",G17=""),"",F17*G17)</f>
         <v>21</v>
       </c>
       <c r="I17" s="14"/>
@@ -3289,7 +3306,7 @@
         <v>7</v>
       </c>
       <c r="H18" s="16" t="n">
-        <f aca="false">IF(F18="","",F18*G18)</f>
+        <f aca="false">IF(OR(F18="",G18=""),"",F18*G18)</f>
         <v>14</v>
       </c>
       <c r="I18" s="14"/>
@@ -3318,7 +3335,7 @@
         <v>7</v>
       </c>
       <c r="H19" s="16" t="n">
-        <f aca="false">IF(F19="","",F19*G19)</f>
+        <f aca="false">IF(OR(F19="",G19=""),"",F19*G19)</f>
         <v>35</v>
       </c>
       <c r="I19" s="14"/>
@@ -3347,7 +3364,7 @@
         <v>11</v>
       </c>
       <c r="H20" s="16" t="n">
-        <f aca="false">IF(F20="","",F20*G20)</f>
+        <f aca="false">IF(OR(F20="",G20=""),"",F20*G20)</f>
         <v>22</v>
       </c>
       <c r="I20" s="14"/>
@@ -3376,7 +3393,7 @@
         <v>7</v>
       </c>
       <c r="H21" s="16" t="n">
-        <f aca="false">IF(F21="","",F21*G21)</f>
+        <f aca="false">IF(OR(F21="",G21=""),"",F21*G21)</f>
         <v>14</v>
       </c>
       <c r="I21" s="14"/>
@@ -3405,7 +3422,7 @@
         <v>11</v>
       </c>
       <c r="H22" s="16" t="n">
-        <f aca="false">IF(F22="","",F22*G22)</f>
+        <f aca="false">IF(OR(F22="",G22=""),"",F22*G22)</f>
         <v>22</v>
       </c>
       <c r="I22" s="14"/>
@@ -3434,7 +3451,7 @@
         <v>11</v>
       </c>
       <c r="H23" s="16" t="n">
-        <f aca="false">IF(F23="","",F23*G23)</f>
+        <f aca="false">IF(OR(F23="",G23=""),"",F23*G23)</f>
         <v>11</v>
       </c>
       <c r="I23" s="14"/>
@@ -3463,7 +3480,7 @@
         <v>11</v>
       </c>
       <c r="H24" s="16" t="n">
-        <f aca="false">IF(F24="","",F24*G24)</f>
+        <f aca="false">IF(OR(F24="",G24=""),"",F24*G24)</f>
         <v>66</v>
       </c>
       <c r="I24" s="14"/>
@@ -3492,7 +3509,7 @@
         <v>7</v>
       </c>
       <c r="H25" s="16" t="n">
-        <f aca="false">IF(F25="","",F25*G25)</f>
+        <f aca="false">IF(OR(F25="",G25=""),"",F25*G25)</f>
         <v>70</v>
       </c>
       <c r="I25" s="14"/>
@@ -3521,7 +3538,7 @@
         <v>7</v>
       </c>
       <c r="H26" s="16" t="n">
-        <f aca="false">IF(F26="","",F26*G26)</f>
+        <f aca="false">IF(OR(F26="",G26=""),"",F26*G26)</f>
         <v>21</v>
       </c>
       <c r="I26" s="14"/>
@@ -3550,7 +3567,7 @@
         <v>7</v>
       </c>
       <c r="H27" s="16" t="n">
-        <f aca="false">IF(F27="","",F27*G27)</f>
+        <f aca="false">IF(OR(F27="",G27=""),"",F27*G27)</f>
         <v>21</v>
       </c>
       <c r="I27" s="14"/>
@@ -3674,7 +3691,7 @@
         <v>11</v>
       </c>
       <c r="H5" s="11" t="n">
-        <f aca="false">IF(F5="","",F5*G5)</f>
+        <f aca="false">IF(OR(F5="",G5=""),"",F5*G5)</f>
         <v>187</v>
       </c>
       <c r="I5" s="8"/>
@@ -3714,7 +3731,7 @@
         <v>11</v>
       </c>
       <c r="H6" s="11" t="n">
-        <f aca="false">IF(F6="","",F6*G6)</f>
+        <f aca="false">IF(OR(F6="",G6=""),"",F6*G6)</f>
         <v>44</v>
       </c>
       <c r="I6" s="8"/>
@@ -3754,7 +3771,7 @@
         <v>11</v>
       </c>
       <c r="H7" s="11" t="n">
-        <f aca="false">IF(F7="","",F7*G7)</f>
+        <f aca="false">IF(OR(F7="",G7=""),"",F7*G7)</f>
         <v>11</v>
       </c>
       <c r="I7" s="8"/>
@@ -3794,7 +3811,7 @@
         <v>22</v>
       </c>
       <c r="H8" s="11" t="n">
-        <f aca="false">IF(F8="","",F8*G8)</f>
+        <f aca="false">IF(OR(F8="",G8=""),"",F8*G8)</f>
         <v>418</v>
       </c>
       <c r="I8" s="8"/>
@@ -3834,7 +3851,7 @@
         <v>22</v>
       </c>
       <c r="H9" s="11" t="n">
-        <f aca="false">IF(F9="","",F9*G9)</f>
+        <f aca="false">IF(OR(F9="",G9=""),"",F9*G9)</f>
         <v>22</v>
       </c>
       <c r="I9" s="8"/>
@@ -3874,7 +3891,7 @@
         <v>22</v>
       </c>
       <c r="H10" s="11" t="n">
-        <f aca="false">IF(F10="","",F10*G10)</f>
+        <f aca="false">IF(OR(F10="",G10=""),"",F10*G10)</f>
         <v>44</v>
       </c>
       <c r="I10" s="8"/>
@@ -3914,7 +3931,7 @@
         <v>22</v>
       </c>
       <c r="H11" s="11" t="n">
-        <f aca="false">IF(F11="","",F11*G11)</f>
+        <f aca="false">IF(OR(F11="",G11=""),"",F11*G11)</f>
         <v>44</v>
       </c>
       <c r="I11" s="8"/>
@@ -3954,7 +3971,7 @@
         <v>11</v>
       </c>
       <c r="H12" s="11" t="n">
-        <f aca="false">IF(F12="","",F12*G12)</f>
+        <f aca="false">IF(OR(F12="",G12=""),"",F12*G12)</f>
         <v>66</v>
       </c>
       <c r="I12" s="8"/>
@@ -3983,7 +4000,7 @@
         <v>11</v>
       </c>
       <c r="H13" s="16" t="n">
-        <f aca="false">IF(F13="","",F13*G13)</f>
+        <f aca="false">IF(OR(F13="",G13=""),"",F13*G13)</f>
         <v>88</v>
       </c>
       <c r="I13" s="14"/>
@@ -4012,7 +4029,7 @@
         <v>46.5</v>
       </c>
       <c r="H14" s="16" t="n">
-        <f aca="false">IF(F14="","",F14*G14)</f>
+        <f aca="false">IF(OR(F14="",G14=""),"",F14*G14)</f>
         <v>372</v>
       </c>
       <c r="I14" s="14"/>
@@ -4041,7 +4058,7 @@
         <v>22</v>
       </c>
       <c r="H15" s="16" t="n">
-        <f aca="false">IF(F15="","",F15*G15)</f>
+        <f aca="false">IF(OR(F15="",G15=""),"",F15*G15)</f>
         <v>176</v>
       </c>
       <c r="I15" s="14"/>
@@ -4070,7 +4087,7 @@
         <v>22</v>
       </c>
       <c r="H16" s="16" t="n">
-        <f aca="false">IF(F16="","",F16*G16)</f>
+        <f aca="false">IF(OR(F16="",G16=""),"",F16*G16)</f>
         <v>176</v>
       </c>
       <c r="I16" s="14"/>
@@ -4099,7 +4116,7 @@
         <v>22</v>
       </c>
       <c r="H17" s="16" t="n">
-        <f aca="false">IF(F17="","",F17*G17)</f>
+        <f aca="false">IF(OR(F17="",G17=""),"",F17*G17)</f>
         <v>44</v>
       </c>
       <c r="I17" s="14"/>
@@ -4128,7 +4145,7 @@
         <v>11</v>
       </c>
       <c r="H18" s="16" t="n">
-        <f aca="false">IF(F18="","",F18*G18)</f>
+        <f aca="false">IF(OR(F18="",G18=""),"",F18*G18)</f>
         <v>22</v>
       </c>
       <c r="I18" s="14"/>
@@ -4157,7 +4174,7 @@
         <v>11</v>
       </c>
       <c r="H19" s="16" t="n">
-        <f aca="false">IF(F19="","",F19*G19)</f>
+        <f aca="false">IF(OR(F19="",G19=""),"",F19*G19)</f>
         <v>77</v>
       </c>
       <c r="I19" s="14"/>
@@ -4186,7 +4203,7 @@
         <v>22</v>
       </c>
       <c r="H20" s="16" t="n">
-        <f aca="false">IF(F20="","",F20*G20)</f>
+        <f aca="false">IF(OR(F20="",G20=""),"",F20*G20)</f>
         <v>66</v>
       </c>
       <c r="I20" s="14"/>
@@ -4215,7 +4232,7 @@
         <v>11</v>
       </c>
       <c r="H21" s="16" t="n">
-        <f aca="false">IF(F21="","",F21*G21)</f>
+        <f aca="false">IF(OR(F21="",G21=""),"",F21*G21)</f>
         <v>33</v>
       </c>
       <c r="I21" s="14"/>
@@ -4244,7 +4261,7 @@
         <v>22</v>
       </c>
       <c r="H22" s="16" t="n">
-        <f aca="false">IF(F22="","",F22*G22)</f>
+        <f aca="false">IF(OR(F22="",G22=""),"",F22*G22)</f>
         <v>22</v>
       </c>
       <c r="I22" s="14"/>
@@ -4273,7 +4290,7 @@
         <v>11</v>
       </c>
       <c r="H23" s="16" t="n">
-        <f aca="false">IF(F23="","",F23*G23)</f>
+        <f aca="false">IF(OR(F23="",G23=""),"",F23*G23)</f>
         <v>22</v>
       </c>
       <c r="I23" s="14"/>
@@ -4302,7 +4319,7 @@
         <v>11</v>
       </c>
       <c r="H24" s="16" t="n">
-        <f aca="false">IF(F24="","",F24*G24)</f>
+        <f aca="false">IF(OR(F24="",G24=""),"",F24*G24)</f>
         <v>11</v>
       </c>
       <c r="I24" s="14"/>
@@ -4331,10 +4348,1023 @@
         <v>11</v>
       </c>
       <c r="H25" s="16" t="n">
-        <f aca="false">IF(F25="","",F25*G25)</f>
+        <f aca="false">IF(OR(F25="",G25=""),"",F25*G25)</f>
         <v>22</v>
       </c>
       <c r="I25" s="14"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:M27"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <f aca="false">SUM(F5:F1000)</f>
+        <v>56</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D2" s="5" t="n">
+        <f aca="false">SUM(H5:H1000)</f>
+        <v>1408</v>
+      </c>
+      <c r="E2" s="20" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="K4" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="L4" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="M4" s="21" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="G5" s="23" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C5,'Bulk Pricing'!$C:$C,D5,'Bulk Pricing'!$D:$D,E5)</f>
+        <v>12</v>
+      </c>
+      <c r="H5" s="11" t="n">
+        <f aca="false">IF(OR(F5="",G5=""),"",F5*G5)</f>
+        <v>36</v>
+      </c>
+      <c r="I5" s="8"/>
+      <c r="K5" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="L5" s="7" t="n">
+        <f aca="false">SUMIFS($F$5:$F$1000,$B$5:$B$1000,K5)</f>
+        <v>1</v>
+      </c>
+      <c r="M5" s="11" t="n">
+        <f aca="false">SUMIFS($H$5:$H$1000,$B$5:$B$1000,K5)</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G6" s="23" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C6,'Bulk Pricing'!$C:$C,D6,'Bulk Pricing'!$D:$D,E6)</f>
+        <v>23.5</v>
+      </c>
+      <c r="H6" s="11" t="n">
+        <f aca="false">IF(OR(F6="",G6=""),"",F6*G6)</f>
+        <v>47</v>
+      </c>
+      <c r="I6" s="8"/>
+      <c r="K6" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="L6" s="7" t="n">
+        <f aca="false">SUMIFS($F$5:$F$1000,$B$5:$B$1000,K6)</f>
+        <v>2</v>
+      </c>
+      <c r="M6" s="11" t="n">
+        <f aca="false">SUMIFS($H$5:$H$1000,$B$5:$B$1000,K6)</f>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F7" s="22" t="n">
+        <v>9</v>
+      </c>
+      <c r="G7" s="23" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C7,'Bulk Pricing'!$C:$C,D7,'Bulk Pricing'!$D:$D,E7)</f>
+        <v>49.5</v>
+      </c>
+      <c r="H7" s="11" t="n">
+        <f aca="false">IF(OR(F7="",G7=""),"",F7*G7)</f>
+        <v>445.5</v>
+      </c>
+      <c r="I7" s="8"/>
+      <c r="K7" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="L7" s="7" t="n">
+        <f aca="false">SUMIFS($F$5:$F$1000,$B$5:$B$1000,K7)</f>
+        <v>8</v>
+      </c>
+      <c r="M7" s="11" t="n">
+        <f aca="false">SUMIFS($H$5:$H$1000,$B$5:$B$1000,K7)</f>
+        <v>143.5</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="23" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C8,'Bulk Pricing'!$C:$C,D8,'Bulk Pricing'!$D:$D,E8)</f>
+        <v>23.5</v>
+      </c>
+      <c r="H8" s="11" t="n">
+        <f aca="false">IF(OR(F8="",G8=""),"",F8*G8)</f>
+        <v>23.5</v>
+      </c>
+      <c r="I8" s="8"/>
+      <c r="K8" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="L8" s="7" t="n">
+        <f aca="false">SUMIFS($F$5:$F$1000,$B$5:$B$1000,K8)</f>
+        <v>11</v>
+      </c>
+      <c r="M8" s="11" t="n">
+        <f aca="false">SUMIFS($H$5:$H$1000,$B$5:$B$1000,K8)</f>
+        <v>315.5</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F9" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="23" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C9,'Bulk Pricing'!$C:$C,D9,'Bulk Pricing'!$D:$D,E9)</f>
+        <v>12</v>
+      </c>
+      <c r="H9" s="11" t="n">
+        <f aca="false">IF(OR(F9="",G9=""),"",F9*G9)</f>
+        <v>12</v>
+      </c>
+      <c r="I9" s="8"/>
+      <c r="K9" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="L9" s="7" t="n">
+        <f aca="false">SUMIFS($F$5:$F$1000,$B$5:$B$1000,K9)</f>
+        <v>1</v>
+      </c>
+      <c r="M9" s="11" t="n">
+        <f aca="false">SUMIFS($H$5:$H$1000,$B$5:$B$1000,K9)</f>
+        <v>23.5</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F10" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="G10" s="23" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C10,'Bulk Pricing'!$C:$C,D10,'Bulk Pricing'!$D:$D,E10)</f>
+        <v>12</v>
+      </c>
+      <c r="H10" s="11" t="n">
+        <f aca="false">IF(OR(F10="",G10=""),"",F10*G10)</f>
+        <v>48</v>
+      </c>
+      <c r="I10" s="8"/>
+      <c r="K10" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="L10" s="7" t="n">
+        <f aca="false">SUMIFS($F$5:$F$1000,$B$5:$B$1000,K10)</f>
+        <v>18</v>
+      </c>
+      <c r="M10" s="11" t="n">
+        <f aca="false">SUMIFS($H$5:$H$1000,$B$5:$B$1000,K10)</f>
+        <v>585.5</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F11" s="22" t="n">
+        <v>6</v>
+      </c>
+      <c r="G11" s="23" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C11,'Bulk Pricing'!$C:$C,D11,'Bulk Pricing'!$D:$D,E11)</f>
+        <v>23.5</v>
+      </c>
+      <c r="H11" s="11" t="n">
+        <f aca="false">IF(OR(F11="",G11=""),"",F11*G11)</f>
+        <v>141</v>
+      </c>
+      <c r="I11" s="8"/>
+      <c r="K11" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="L11" s="7" t="n">
+        <f aca="false">SUMIFS($F$5:$F$1000,$B$5:$B$1000,K11)</f>
+        <v>15</v>
+      </c>
+      <c r="M11" s="11" t="n">
+        <f aca="false">SUMIFS($H$5:$H$1000,$B$5:$B$1000,K11)</f>
+        <v>278</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F12" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="23" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C12,'Bulk Pricing'!$C:$C,D12,'Bulk Pricing'!$D:$D,E12)</f>
+        <v>23.5</v>
+      </c>
+      <c r="H12" s="11" t="n">
+        <f aca="false">IF(OR(F12="",G12=""),"",F12*G12)</f>
+        <v>23.5</v>
+      </c>
+      <c r="I12" s="8"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F13" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G13" s="23" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C13,'Bulk Pricing'!$C:$C,D13,'Bulk Pricing'!$D:$D,E13)</f>
+        <v>23.5</v>
+      </c>
+      <c r="H13" s="11" t="n">
+        <f aca="false">IF(OR(F13="",G13=""),"",F13*G13)</f>
+        <v>47</v>
+      </c>
+      <c r="I13" s="8"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F14" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="G14" s="23" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C14,'Bulk Pricing'!$C:$C,D14,'Bulk Pricing'!$D:$D,E14)</f>
+        <v>12</v>
+      </c>
+      <c r="H14" s="11" t="n">
+        <f aca="false">IF(OR(F14="",G14=""),"",F14*G14)</f>
+        <v>48</v>
+      </c>
+      <c r="I14" s="8"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D15" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F15" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="23" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C15,'Bulk Pricing'!$C:$C,D15,'Bulk Pricing'!$D:$D,E15)</f>
+        <v>23.5</v>
+      </c>
+      <c r="H15" s="11" t="n">
+        <f aca="false">IF(OR(F15="",G15=""),"",F15*G15)</f>
+        <v>23.5</v>
+      </c>
+      <c r="I15" s="8"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D16" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F16" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" s="23" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C16,'Bulk Pricing'!$C:$C,D16,'Bulk Pricing'!$D:$D,E16)</f>
+        <v>23.5</v>
+      </c>
+      <c r="H16" s="11" t="n">
+        <f aca="false">IF(OR(F16="",G16=""),"",F16*G16)</f>
+        <v>23.5</v>
+      </c>
+      <c r="I16" s="8"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D17" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F17" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="23" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C17,'Bulk Pricing'!$C:$C,D17,'Bulk Pricing'!$D:$D,E17)</f>
+        <v>12</v>
+      </c>
+      <c r="H17" s="11" t="n">
+        <f aca="false">IF(OR(F17="",G17=""),"",F17*G17)</f>
+        <v>12</v>
+      </c>
+      <c r="I17" s="8"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D18" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F18" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="23" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C18,'Bulk Pricing'!$C:$C,D18,'Bulk Pricing'!$D:$D,E18)</f>
+        <v>12</v>
+      </c>
+      <c r="H18" s="11" t="n">
+        <f aca="false">IF(OR(F18="",G18=""),"",F18*G18)</f>
+        <v>12</v>
+      </c>
+      <c r="I18" s="8"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C19" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="D19" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="E19" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F19" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G19" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C19,'Bulk Pricing'!$C:$C,D19,'Bulk Pricing'!$D:$D,E19)</f>
+        <v>25</v>
+      </c>
+      <c r="H19" s="16" t="n">
+        <f aca="false">IF(OR(F19="",G19=""),"",F19*G19)</f>
+        <v>50</v>
+      </c>
+      <c r="I19" s="14"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="13" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="C20" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="D20" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="E20" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F20" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G20" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C20,'Bulk Pricing'!$C:$C,D20,'Bulk Pricing'!$D:$D,E20)</f>
+        <v>25</v>
+      </c>
+      <c r="H20" s="16" t="n">
+        <f aca="false">IF(OR(F20="",G20=""),"",F20*G20)</f>
+        <v>50</v>
+      </c>
+      <c r="I20" s="14"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="C21" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="D21" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="E21" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F21" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C21,'Bulk Pricing'!$C:$C,D21,'Bulk Pricing'!$D:$D,E21)</f>
+        <v>25</v>
+      </c>
+      <c r="H21" s="16" t="n">
+        <f aca="false">IF(OR(F21="",G21=""),"",F21*G21)</f>
+        <v>25</v>
+      </c>
+      <c r="I21" s="14"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="13" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C22" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="D22" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E22" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F22" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="G22" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C22,'Bulk Pricing'!$C:$C,D22,'Bulk Pricing'!$D:$D,E22)</f>
+        <v>13.5</v>
+      </c>
+      <c r="H22" s="16" t="n">
+        <f aca="false">IF(OR(F22="",G22=""),"",F22*G22)</f>
+        <v>40.5</v>
+      </c>
+      <c r="I22" s="14"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="13" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C23" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="D23" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="E23" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F23" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C23,'Bulk Pricing'!$C:$C,D23,'Bulk Pricing'!$D:$D,E23)</f>
+        <v>25</v>
+      </c>
+      <c r="H23" s="16" t="n">
+        <f aca="false">IF(OR(F23="",G23=""),"",F23*G23)</f>
+        <v>25</v>
+      </c>
+      <c r="I23" s="14"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="C24" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="D24" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E24" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F24" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="G24" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C24,'Bulk Pricing'!$C:$C,D24,'Bulk Pricing'!$D:$D,E24)</f>
+        <v>13.5</v>
+      </c>
+      <c r="H24" s="16" t="n">
+        <f aca="false">IF(OR(F24="",G24=""),"",F24*G24)</f>
+        <v>67.5</v>
+      </c>
+      <c r="I24" s="14"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="13" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="C25" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="D25" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="E25" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="F25" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C25,'Bulk Pricing'!$C:$C,D25,'Bulk Pricing'!$D:$D,E25)</f>
+        <v>25</v>
+      </c>
+      <c r="H25" s="16" t="n">
+        <f aca="false">IF(OR(F25="",G25=""),"",F25*G25)</f>
+        <v>25</v>
+      </c>
+      <c r="I25" s="14"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="13" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C26" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="D26" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="E26" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="F26" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C26,'Bulk Pricing'!$C:$C,D26,'Bulk Pricing'!$D:$D,E26)</f>
+        <v>25</v>
+      </c>
+      <c r="H26" s="16" t="n">
+        <f aca="false">IF(OR(F26="",G26=""),"",F26*G26)</f>
+        <v>25</v>
+      </c>
+      <c r="I26" s="14"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="13" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C27" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="D27" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="E27" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="F27" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="G27" s="24" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C27,'Bulk Pricing'!$C:$C,D27,'Bulk Pricing'!$D:$D,E27)</f>
+        <v>52.5</v>
+      </c>
+      <c r="H27" s="16" t="n">
+        <f aca="false">IF(OR(F27="",G27=""),"",F27*G27)</f>
+        <v>157.5</v>
+      </c>
+      <c r="I27" s="14"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:M6"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <f aca="false">SUM(F5:F1000)</f>
+        <v>17</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D2" s="5" t="n">
+        <f aca="false">SUM(H5:H1000)</f>
+        <v>1084.91</v>
+      </c>
+      <c r="E2" s="20" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="K4" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="L4" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="M4" s="21" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>32</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="G5" s="23" t="n">
+        <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C5,'Bulk Pricing'!$C:$C,D5,'Bulk Pricing'!$D:$D,E5)</f>
+        <v>107.5</v>
+      </c>
+      <c r="H5" s="11" t="n">
+        <f aca="false">IF(OR(F5="",G5=""),"",F5*G5)</f>
+        <v>860</v>
+      </c>
+      <c r="I5" s="8"/>
+      <c r="K5" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="L5" s="7" t="n">
+        <f aca="false">SUMIFS($F$5:$F$1000,$B$5:$B$1000,K5)</f>
+        <v>9</v>
+      </c>
+      <c r="M5" s="11" t="n">
+        <f aca="false">SUMIFS($H$5:$H$1000,$B$5:$B$1000,K5)</f>
+        <v>224.91</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="D6" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>9</v>
+      </c>
+      <c r="G6" s="10" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="H6" s="16" t="n">
+        <f aca="false">IF(OR(F6="",G6=""),"",F6*G6)</f>
+        <v>224.91</v>
+      </c>
+      <c r="I6" s="14"/>
+      <c r="K6" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="L6" s="7" t="n">
+        <f aca="false">SUMIFS($F$5:$F$1000,$B$5:$B$1000,K6)</f>
+        <v>8</v>
+      </c>
+      <c r="M6" s="11" t="n">
+        <f aca="false">SUMIFS($H$5:$H$1000,$B$5:$B$1000,K6)</f>
+        <v>860</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Price 32GB DDR4-3200 server RDIMMs at $200
Lot 4 total now $1,824.91.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BFknSiXKDWdHdxsn9XQpko
</commit_message>
<xml_diff>
--- a/ram_bulk_pricing.xlsx
+++ b/ram_bulk_pricing.xlsx
@@ -145,7 +145,7 @@
     <t xml:space="preserve">4GB: desktop, laptop and server are all the same price for a given speed.</t>
   </si>
   <si>
-    <t xml:space="preserve">Server matches desktop/laptop prices, except 8GB DDR4-2133/2400 server ($20) and DDR4-2133 16/32GB server below.</t>
+    <t xml:space="preserve">Server matches desktop/laptop prices, except 8GB DDR4-2133/2400 server ($20), 32GB DDR4-3200 server ($200), and DDR4-2133 16/32GB server below.</t>
   </si>
   <si>
     <t xml:space="preserve">Server DDR4-2133: 16GB stick = 2 x the 8GB server price + $2.50; 32GB = 2 x the 16GB server price + $2.50.</t>
@@ -2566,11 +2566,11 @@
         <v>17</v>
       </c>
       <c r="E64" s="10" t="n">
-        <v>107.5</v>
+        <v>200</v>
       </c>
       <c r="F64" s="16" t="n">
         <f aca="false">IF(E64="","",E64/C64)</f>
-        <v>3.359375</v>
+        <v>6.25</v>
       </c>
       <c r="G64" s="12"/>
       <c r="H64" s="16" t="str">
@@ -5243,7 +5243,7 @@
       </c>
       <c r="D2" s="5" t="n">
         <f aca="false">SUM(H5:H1000)</f>
-        <v>1084.91</v>
+        <v>1824.91</v>
       </c>
       <c r="E2" s="20" t="s">
         <v>46</v>
@@ -5308,11 +5308,11 @@
       </c>
       <c r="G5" s="23" t="n">
         <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C5,'Bulk Pricing'!$C:$C,D5,'Bulk Pricing'!$D:$D,E5)</f>
-        <v>107.5</v>
+        <v>200</v>
       </c>
       <c r="H5" s="11" t="n">
         <f aca="false">IF(OR(F5="",G5=""),"",F5*G5)</f>
-        <v>860</v>
+        <v>1600</v>
       </c>
       <c r="I5" s="8"/>
       <c r="K5" s="8" t="s">
@@ -5363,7 +5363,7 @@
       </c>
       <c r="M6" s="11" t="n">
         <f aca="false">SUMIFS($H$5:$H$1000,$B$5:$B$1000,K6)</f>
-        <v>860</v>
+        <v>1600</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Split lot 4 into server (lot 4) and Cisco (lot 5) listings
Lot 4: 8x SK Hynix 32GB DDR4-3200 RDIMM, $1,600.
Lot 5: 9x Cisco 4GB DRAM, $224.91.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BFknSiXKDWdHdxsn9XQpko
</commit_message>
<xml_diff>
--- a/ram_bulk_pricing.xlsx
+++ b/ram_bulk_pricing.xlsx
@@ -13,7 +13,8 @@
     <sheet name="Lot 1 - DDR3" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Lot 2 - DDR4" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Lot 3 - DDR4 2666-3200" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Lot 4 - Server &amp; Cisco" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Lot 4 - Server" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Lot 5 - Cisco" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Bulk Pricing'!$A$4:$I$64</definedName>
@@ -50,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="531" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="69">
   <si>
     <t xml:space="preserve">RAM Bulk Buyer Pricing (all brands, non-gaming)</t>
   </si>
@@ -247,7 +248,10 @@
     <t xml:space="preserve">Forza</t>
   </si>
   <si>
-    <t xml:space="preserve">eBay Bulk Lot 4 - Server &amp; Cisco (all tested)</t>
+    <t xml:space="preserve">eBay Bulk Lot 4 - Server RAM (all tested)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">eBay Bulk Lot 5 - Cisco DRAM (all tested)</t>
   </si>
   <si>
     <t xml:space="preserve">Cisco</t>
@@ -5208,7 +5212,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -5236,14 +5240,14 @@
       </c>
       <c r="B2" s="2" t="n">
         <f aca="false">SUM(F5:F1000)</f>
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>45</v>
       </c>
       <c r="D2" s="5" t="n">
         <f aca="false">SUM(H5:H1000)</f>
-        <v>1824.91</v>
+        <v>1600</v>
       </c>
       <c r="E2" s="20" t="s">
         <v>46</v>
@@ -5316,7 +5320,141 @@
       </c>
       <c r="I5" s="8"/>
       <c r="K5" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="L5" s="7" t="n">
+        <f aca="false">SUMIFS($F$5:$F$1000,$B$5:$B$1000,K5)</f>
+        <v>8</v>
+      </c>
+      <c r="M5" s="11" t="n">
+        <f aca="false">SUMIFS($H$5:$H$1000,$B$5:$B$1000,K5)</f>
+        <v>1600</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:M5"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
         <v>66</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <f aca="false">SUM(F5:F1000)</f>
+        <v>9</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D2" s="5" t="n">
+        <f aca="false">SUM(H5:H1000)</f>
+        <v>224.91</v>
+      </c>
+      <c r="E2" s="20" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="K4" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="L4" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="M4" s="21" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>9</v>
+      </c>
+      <c r="G5" s="10" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="H5" s="11" t="n">
+        <f aca="false">IF(OR(F5="",G5=""),"",F5*G5)</f>
+        <v>224.91</v>
+      </c>
+      <c r="I5" s="8"/>
+      <c r="K5" s="8" t="s">
+        <v>67</v>
       </c>
       <c r="L5" s="7" t="n">
         <f aca="false">SUMIFS($F$5:$F$1000,$B$5:$B$1000,K5)</f>
@@ -5325,45 +5463,6 @@
       <c r="M5" s="11" t="n">
         <f aca="false">SUMIFS($H$5:$H$1000,$B$5:$B$1000,K5)</f>
         <v>224.91</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="D6" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="E6" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="F6" s="22" t="n">
-        <v>9</v>
-      </c>
-      <c r="G6" s="10" t="n">
-        <v>24.99</v>
-      </c>
-      <c r="H6" s="16" t="n">
-        <f aca="false">IF(OR(F6="",G6=""),"",F6*G6)</f>
-        <v>224.91</v>
-      </c>
-      <c r="I6" s="14"/>
-      <c r="K6" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="L6" s="7" t="n">
-        <f aca="false">SUMIFS($F$5:$F$1000,$B$5:$B$1000,K6)</f>
-        <v>8</v>
-      </c>
-      <c r="M6" s="11" t="n">
-        <f aca="false">SUMIFS($H$5:$H$1000,$B$5:$B$1000,K6)</f>
-        <v>1600</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Correct lot 4 server RAM to DDR4-2666 (PC4-2666V)
Moves the $200 32GB server price from DDR4-3200 to DDR4-2666;
3200 32GB server reverts to matching desktop/laptop.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BFknSiXKDWdHdxsn9XQpko
</commit_message>
<xml_diff>
--- a/ram_bulk_pricing.xlsx
+++ b/ram_bulk_pricing.xlsx
@@ -146,7 +146,7 @@
     <t xml:space="preserve">4GB: desktop, laptop and server are all the same price for a given speed.</t>
   </si>
   <si>
-    <t xml:space="preserve">Server matches desktop/laptop prices, except 8GB DDR4-2133/2400 server ($20), 32GB DDR4-3200 server ($200), and DDR4-2133 16/32GB server below.</t>
+    <t xml:space="preserve">Server matches desktop/laptop prices, except 8GB DDR4-2133/2400 server ($20), 32GB DDR4-2666 server ($200), and DDR4-2133 16/32GB server below.</t>
   </si>
   <si>
     <t xml:space="preserve">Server DDR4-2133: 16GB stick = 2 x the 8GB server price + $2.50; 32GB = 2 x the 16GB server price + $2.50.</t>
@@ -2234,11 +2234,11 @@
         <v>17</v>
       </c>
       <c r="E52" s="10" t="n">
-        <v>101.5</v>
+        <v>200</v>
       </c>
       <c r="F52" s="11" t="n">
         <f aca="false">IF(E52="","",E52/C52)</f>
-        <v>3.171875</v>
+        <v>6.25</v>
       </c>
       <c r="G52" s="12"/>
       <c r="H52" s="11" t="str">
@@ -2570,11 +2570,11 @@
         <v>17</v>
       </c>
       <c r="E64" s="10" t="n">
-        <v>200</v>
+        <v>107.5</v>
       </c>
       <c r="F64" s="16" t="n">
         <f aca="false">IF(E64="","",E64/C64)</f>
-        <v>6.25</v>
+        <v>3.359375</v>
       </c>
       <c r="G64" s="12"/>
       <c r="H64" s="16" t="str">
@@ -5299,7 +5299,7 @@
         <v>56</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D5" s="9" t="n">
         <v>32</v>

</xml_diff>

<commit_message>
Raise DDR4 single-listing prices from sold comps; relist lot 4 at $1,400
Inventory suggested/floor prices updated per ddr4_price_review.md.
Lot 4 (8x 32GB DDR4-2666 server) order was cancelled; now $175/stick.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BFknSiXKDWdHdxsn9XQpko
</commit_message>
<xml_diff>
--- a/ram_bulk_pricing.xlsx
+++ b/ram_bulk_pricing.xlsx
@@ -146,7 +146,7 @@
     <t xml:space="preserve">4GB: desktop, laptop and server are all the same price for a given speed.</t>
   </si>
   <si>
-    <t xml:space="preserve">Server matches desktop/laptop prices, except 8GB DDR4-2133/2400 server ($20), 32GB DDR4-2666 server ($200), and DDR4-2133 16/32GB server below.</t>
+    <t xml:space="preserve">Server matches desktop/laptop prices, except 8GB DDR4-2133/2400 server ($20), 32GB DDR4-2666 server ($175), and DDR4-2133 16/32GB server below.</t>
   </si>
   <si>
     <t xml:space="preserve">Server DDR4-2133: 16GB stick = 2 x the 8GB server price + $2.50; 32GB = 2 x the 16GB server price + $2.50.</t>
@@ -2234,11 +2234,11 @@
         <v>17</v>
       </c>
       <c r="E52" s="10" t="n">
-        <v>200</v>
+        <v>175</v>
       </c>
       <c r="F52" s="11" t="n">
         <f aca="false">IF(E52="","",E52/C52)</f>
-        <v>6.25</v>
+        <v>5.46875</v>
       </c>
       <c r="G52" s="12"/>
       <c r="H52" s="11" t="str">
@@ -5247,7 +5247,7 @@
       </c>
       <c r="D2" s="5" t="n">
         <f aca="false">SUM(H5:H1000)</f>
-        <v>1600</v>
+        <v>1400</v>
       </c>
       <c r="E2" s="20" t="s">
         <v>46</v>
@@ -5312,11 +5312,11 @@
       </c>
       <c r="G5" s="23" t="n">
         <f aca="false">SUMIFS('Bulk Pricing'!$E:$E,'Bulk Pricing'!$B:$B,C5,'Bulk Pricing'!$C:$C,D5,'Bulk Pricing'!$D:$D,E5)</f>
-        <v>200</v>
+        <v>175</v>
       </c>
       <c r="H5" s="11" t="n">
         <f aca="false">IF(OR(F5="",G5=""),"",F5*G5)</f>
-        <v>1600</v>
+        <v>1400</v>
       </c>
       <c r="I5" s="8"/>
       <c r="K5" s="8" t="s">
@@ -5328,7 +5328,7 @@
       </c>
       <c r="M5" s="11" t="n">
         <f aca="false">SUMIFS($H$5:$H$1000,$B$5:$B$1000,K5)</f>
-        <v>1600</v>
+        <v>1400</v>
       </c>
     </row>
   </sheetData>

</xml_diff>